<commit_message>
refactor(day22): streamline deliverables, apply Times New Roman 13pt format, and refine professional language
</commit_message>
<xml_diff>
--- a/MinhNQ_Day22_model.xlsx
+++ b/MinhNQ_Day22_model.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Projects\AI_Thuc_chien_Khoa_IV\02_THUC_HANH\Track1_Day22_2A202602432_NinhQuangMinh\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2A0401F-28EF-467B-B6E2-52200769BE5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FF2CA6F-632A-4D13-A36F-B1D5024EB0B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -169,7 +169,7 @@
     <t>1 job của bạn là gì?</t>
   </si>
   <si>
-    <t>1 ca tiếp nhận &amp; phân tầng triệu chứng bệnh nhân hoàn thành (bệnh nhân nhận kết quả triage sơ bộ có phân tầng khẩn cấp ESI + hướng dẫn đặt khám, hoặc được điều dưỡng trực xác nhận/tiếp nhận)</t>
+    <t>1 ca tiếp nhận và phân tầng triệu chứng bệnh nhân (bệnh nhân nhận kết quả sơ loại ESI, hướng dẫn đặt chuyên khoa hoặc điều dưỡng tiếp nhận).</t>
   </si>
   <si>
     <t>Phải là thứ KHÁCH coi là giá trị — không phải '1 request'</t>
@@ -691,7 +691,7 @@
     <t>Usage / Outcome</t>
   </si>
   <si>
-    <t>$2,00 / conversation ($0,10/action)</t>
+    <t>$2,00 / conversation</t>
   </si>
   <si>
     <t>https://www.salesforce.com/agentforce/pricing/</t>
@@ -709,25 +709,25 @@
     <t>Nếu KHÁC gợi ý — lý do thị trường là gì?</t>
   </si>
   <si>
-    <t>Y tế là ngành high-stakes, rủi ro cao. Bệnh viện không chấp nhận thanh toán theo lượt token (khó dự toán) và nhà cung cấp không thể chỉ bán Outcome thuần nếu không có phí duy trì bảo mật HIPAA/NĐ13. Mô hình Hybrid ($300 phí nền hạ tầng/tháng/cơ sở + $0,79/ca triage hoàn thành) cân bằng tối ưu rủi ro hai bên.</t>
+    <t>Y tế là ngành rủi ro cao. Khách hàng không chấp nhận thanh toán theo token do khó dự toán ngân sách; nhà cung cấp không thể chỉ thu theo outcome nếu không có phí duy trì hạ tầng tuân thủ bảo mật dữ liệu y tế. Mô hình Hybrid ($300 phí nền/tháng/cơ sở + $0,79/ca hoàn thành) giúp cân bằng rủi ro cho cả hai bên.</t>
   </si>
   <si>
     <t>Decision Note — câu 1: tôi chọn đơn vị nào?</t>
   </si>
   <si>
-    <t>Đơn vị tính tiền: Hybrid — Phí nền duy trì hạ tầng &amp; bảo mật y tế ($300/tháng/cơ sở) + $0,79 / ca tiếp nhận &amp; phân tầng hoàn thành (Qualified Clinical Triage Outcome).</t>
+    <t>Đơn vị tính tiền: Hybrid — Phí nền duy trì hạ tầng ($300/tháng/cơ sở) + $0,79/ca tiếp nhận và phân tầng hoàn thành.</t>
   </si>
   <si>
     <t>Decision Note — câu 2: bằng chứng Attribution / Autonomy?</t>
   </si>
   <si>
-    <t>Attribution đạt 9/10 nhờ log chi tiết session ID và mã phân tầng ESI nối trực tiếp vào hệ thống đặt hẹn; Autonomy đạt 6/10 do quy chuẩn an toàn y khoa bắt buộc có điều dưỡng trực xác nhận ca cờ đỏ (Red Flag) và audit 6% ngẫu nhiên.</t>
+    <t>Attribution đạt 9/10 do lưu vết đầy đủ session ID và mã ESI vào hệ thống đặt hẹn; Autonomy đạt 6/10 do quy trình y tế bắt buộc có điều dưỡng trực xác nhận ca cờ đỏ (Red Flag) và kiểm toán 6% ca ngẫu nhiên.</t>
   </si>
   <si>
     <t>Decision Note — câu 3: mô hình này lỗ trong tình huống nào?</t>
   </si>
   <si>
-    <t>Mô hình này lỗ khi tỷ lệ Containment tụt dưới 70,3% (quá nhiều ca escalate sang điều dưỡng trực với chi phí nhân sự $7/giờ) hoặc giá API LLM tăng đột biến mà không áp dụng prompt caching.</t>
+    <t>Mô hình lỗ khi tỷ lệ Containment giảm dưới 70,3% (nhiều ca phải chuyển sang điều dưỡng xử lý làm tăng chi phí nhân sự) hoặc chi phí token tăng do mất cache.</t>
   </si>
   <si>
     <t>TAB 4 — CHANNEL FIT &amp; AFFORDABILITY TEST</t>
@@ -868,7 +868,7 @@
     <t>Nếu Partner-Led: TÊN CÔNG TY partner</t>
   </si>
   <si>
-    <t>Hệ thống Y tế Vinmec (Vinmec Healthcare System)</t>
+    <t>Hệ thống Y tế Vinmec</t>
   </si>
   <si>
     <t>'Các nền tảng trong ngành' = chưa có kênh</t>
@@ -883,13 +883,13 @@
     <t>Bạn mang lại giá trị gì cho partner?</t>
   </si>
   <si>
-    <t>Mang lại giải pháp phân luồng tự động 24/7 giúp Vinmec giải tỏa 80% áp lực tổng đài trực đêm, giảm thời gian chờ tiếp nhận tại khoa khám bệnh từ 15 phút xuống 2 phút, và tăng tỷ lệ chuyển đổi bệnh nhân đặt khám đúng chuyên khoa.</t>
+    <t>Cung cấp giải pháp phân luồng tự động 24/7 giúp Vinmec giảm tải tổng đài ban đêm, rút ngắn thời gian chờ tại quầy tiếp đón từ 15 phút xuống 2 phút và tăng tỷ lệ đặt hẹn đúng chuyên khoa.</t>
   </si>
   <si>
     <t>Nếu rơi vào vùng không khả thi — lối thoát nào?</t>
   </si>
   <si>
-    <t>Bypass bài toán CAC cao bằng mô hình Partner-Led: Nhúng trực tiếp vào Zalo OA Vinmec và Ứng dụng MyVinmec có sẵn hàng trăm nghìn người dùng, chia sẻ doanh thu giá trị gia tăng thay vì tự đốt tiền chạy quảng cáo tìm bệnh nhân.</t>
+    <t>Chuyển sang Partner-Led để tận dụng tệp bệnh nhân sẵn có trên ứng dụng MyVinmec và Zalo OA Vinmec, chia sẻ doanh thu thay vì chịu chi phí CAC bán hàng trực tiếp quá cao.</t>
   </si>
   <si>
     <t>Giảm giá để tự phục vụ / tăng giá + service / Partner-Led</t>
@@ -907,25 +907,25 @@
     <t>MẤY GIỜ khách đau nhất?</t>
   </si>
   <si>
-    <t>21:30 – 23:30 đêm (ngoài giờ hành chính, phòng khám tư đóng cửa)</t>
+    <t>21:30 – 23:30 (ngoài giờ hành chính, phòng khám ngoại trú đóng cửa)</t>
   </si>
   <si>
     <t>Lúc đó họ ĐANG LÀM GÌ?</t>
   </si>
   <si>
-    <t>Bệnh nhân hoặc người nhà lo lắng vì triệu chứng bất thường (sốt, đau ngực, khó thở, dị ứng), băn khoăn không biết có cần nhập viện cấp cứu ngay trong đêm hay đợi sáng mai đi khám</t>
+    <t>Người bệnh hoặc thân nhân lo lắng khi xuất hiện triệu chứng bất thường, cần xác định mức độ khẩn cấp để quyết định đi cấp cứu hay chờ khám sáng hôm sau</t>
   </si>
   <si>
     <t>Họ đang DÙNG APP / KÊNH NÀO?</t>
   </si>
   <si>
-    <t>Zalo tìm kiếm Zalo OA Vinmec hoặc mở Ứng dụng MyVinmec trên điện thoại</t>
+    <t>Zalo Official Account của Vinmec hoặc ứng dụng MyVinmec</t>
   </si>
   <si>
     <t>→ Điểm nhúng cụ thể của bạn</t>
   </si>
   <si>
-    <t>Widget 'Sơ loại triệu chứng 24/7' nhúng trực tiếp trong Zalo OA Vinmec và mục Khám bệnh trên App MyVinmec (Zero new tabs — không bắt tải app mới)</t>
+    <t>Tính năng 'Sơ loại triệu chứng 24/7' tích hợp trong menu Zalo OA Vinmec và ứng dụng MyVinmec</t>
   </si>
   <si>
     <t>Một bề mặt tích hợp có tên, không phải 'website của chúng tôi'</t>
@@ -946,85 +946,85 @@
     <t>Kênh sử dụng</t>
   </si>
   <si>
-    <t>Partner-Led (Pilot nội bộ tại BVĐKQT Vinmec Times City)</t>
-  </si>
-  <si>
-    <t>Partner-Led (Mở rộng toàn bộ 7 bệnh viện Vinmec trên toàn quốc)</t>
-  </si>
-  <si>
-    <t>Partner-Led &amp; Mid-market Inbound (Mở rộng sang các hệ thống y tế tư nhân khác)</t>
+    <t>Partner-Led (Pilot tại BV Vinmec Times City)</t>
+  </si>
+  <si>
+    <t>Partner-Led (Mở rộng 7 BV và 3 PK Vinmec)</t>
+  </si>
+  <si>
+    <t>Partner-Led và Inbound (Mở rộng chuỗi y tế tư nhân khác)</t>
   </si>
   <si>
     <t>Mục tiêu số khách</t>
   </si>
   <si>
-    <t>1 cơ sở pilot (1.500 ca intake/tháng)</t>
-  </si>
-  <si>
-    <t>7 bệnh viện + 3 phòng khám Vinmec (12.000 ca/tháng)</t>
-  </si>
-  <si>
-    <t>3 hệ thống y tế mới (40.000 ca/tháng)</t>
+    <t>1 cơ sở (1.500 ca/tháng)</t>
+  </si>
+  <si>
+    <t>10 cơ sở (12.000 ca/tháng)</t>
+  </si>
+  <si>
+    <t>3 hệ thống mới (40.000 ca/tháng)</t>
   </si>
   <si>
     <t>Việc cụ thể 1</t>
   </si>
   <si>
-    <t>Tích hợp API sơ loại vào Zalo OA Vinmec Times City &amp; Cổng tiếp nhận</t>
-  </si>
-  <si>
-    <t>Chuẩn hóa quy trình tích hợp sâu với HIS/EHR Vinmec và phân bổ lịch khám</t>
-  </si>
-  <si>
-    <t>Đóng gói 'Clinical Triage Solution Pack' cho các chuỗi bệnh viện tư khác</t>
+    <t>Tích hợp API sơ loại vào Zalo OA và cổng tiếp nhận</t>
+  </si>
+  <si>
+    <t>Tích hợp sâu hệ thống HIS/EHR và phân bổ lịch khám</t>
+  </si>
+  <si>
+    <t>Đóng gói giải pháp tích hợp cho các hệ thống bệnh viện khác</t>
   </si>
   <si>
     <t>Việc cụ thể 2</t>
   </si>
   <si>
-    <t>Phối hợp Hội đồng chuyên môn Vinmec chuẩn hóa 30 bộ kịch bản Red Flags</t>
-  </si>
-  <si>
-    <t>Tối ưu prompt caching, đẩy containment rate lên 78–80%</t>
-  </si>
-  <si>
-    <t>Mở rộng tính năng theo dõi triệu chứng sau khám (post-visit follow-up)</t>
+    <t>Hội đồng chuyên môn chuẩn hóa 30 kịch bản cờ đỏ (Red Flags)</t>
+  </si>
+  <si>
+    <t>Tối ưu hóa prompt caching, nâng containment lên 78–80%</t>
+  </si>
+  <si>
+    <t>Bổ sung tính năng theo dõi triệu chứng sau khám</t>
   </si>
   <si>
     <t>Việc cụ thể 3</t>
   </si>
   <si>
-    <t>Thiết lập quy trình escalate tự động sang trực ban điều dưỡng Cấp cứu (&lt;90s)</t>
-  </si>
-  <si>
-    <t>Xây dựng Executive Dashboard đo Attribution &amp; GM cho Ban Giám đốc Vinmec</t>
-  </si>
-  <si>
-    <t>Hoàn thiện hồ sơ tuân thủ Nghị định 13/2023/NĐ-CP và ISO 27001 y tế</t>
+    <t>Thiết lập luồng chuyển tiếp tự động sang điều dưỡng cấp cứu (&lt;90 giây)</t>
+  </si>
+  <si>
+    <t>Xây dựng dashboard theo dõi Attribution và biên lợi nhuận cho ban lãnh đạo</t>
+  </si>
+  <si>
+    <t>Hoàn thiện hồ sơ tuân thủ Nghị định 13/2023/NĐ-CP và ISO 27001</t>
   </si>
   <si>
     <t>KPI đo được</t>
   </si>
   <si>
-    <t>Containment 75%, CSAT ≥ 4.5/5, 0 sự cố y khoa (zero missed red-flags)</t>
-  </si>
-  <si>
-    <t>Containment ≥ 78%, GM ≥ 71%, thời gian chờ tiếp nhận giảm 80%</t>
-  </si>
-  <si>
-    <t>ARR đạt $380,000, CAC Payback &lt; 8 tháng, NRR &gt; 120%</t>
+    <t>Containment 75%, CSAT ≥ 4,5/5, không có sự cố bỏ sót cờ đỏ</t>
+  </si>
+  <si>
+    <t>Containment ≥ 78%, Gross Margin ≥ 71%, thời gian chờ giảm 80%</t>
+  </si>
+  <si>
+    <t>ARR đạt $380.000, CAC Payback &lt; 8 tháng, NRR &gt; 120%</t>
   </si>
   <si>
     <t>Người chịu trách nhiệm</t>
   </si>
   <si>
-    <t>Ninh Quang Minh (Product Lead) &amp; BS. Trưởng khoa Cấp cứu Vinmec</t>
-  </si>
-  <si>
-    <t>Ninh Quang Minh (Product Lead) &amp; Đội Kỹ thuật Tích hợp HIS Vinmec</t>
-  </si>
-  <si>
-    <t>Head of Business Development &amp; Ninh Quang Minh</t>
+    <t>Ninh Quang Minh (Product Lead) và Bác sĩ Trưởng khoa Cấp cứu</t>
+  </si>
+  <si>
+    <t>Ninh Quang Minh và Đội ngũ Kỹ thuật HIS</t>
+  </si>
+  <si>
+    <t>Đội ngũ Phát triển kinh doanh và Ninh Quang Minh</t>
   </si>
   <si>
     <t>Tháng 1 là giai đoạn HỌC, không phải scale. Kế hoạch 'tháng 1 lấy 200 khách ở 5 ngành' là kế hoạch chưa ai từng thử làm.</t>
@@ -1048,19 +1048,19 @@
     <t xml:space="preserve">1. Eval Results </t>
   </si>
   <si>
-    <t>Bộ test 960 vignette lâm sàng (Nature Medicine protocol): Triage chính xác 94.2%, undertriage ca cấp cứu &lt; 3.5%, 78% giải quyết tự động, 22% escalate an toàn.</t>
-  </si>
-  <si>
-    <t>Ninh Quang Minh · Đã hoàn thành (07/10/2026)</t>
+    <t>Bộ thử nghiệm 960 vignette lâm sàng (Nature Medicine): Độ chính xác 94,2%, undertriage ca cấp cứu &lt; 3,5%, containment 78%, chuyển tiếp điều dưỡng 22%.</t>
+  </si>
+  <si>
+    <t>Ninh Quang Minh · 07/10/2026</t>
   </si>
   <si>
     <t xml:space="preserve">2. Risk Checklist </t>
   </si>
   <si>
-    <t>Bộ giải trình Procurement &amp; Clinical Governance: 100% không hallucinate chẩn đoán (chỉ triage nguy cơ), cam kết Zero Data Retention qua Azure/Anthropic Enterprise, tuân thủ Nghị định 13/2023/NĐ-CP.</t>
-  </si>
-  <si>
-    <t>Ninh Quang Minh · Đã hoàn thành (08/10/2026)</t>
+    <t>Báo cáo Procurement: Guardrail không chẩn đoán xác định, cam kết Zero Data Retention qua Azure/Anthropic Enterprise, lưu trữ tại Private Cloud Vinmec.</t>
+  </si>
+  <si>
+    <t>Ninh Quang Minh · 08/10/2026</t>
   </si>
   <si>
     <t>3. Pilot Report</t>
@@ -1069,10 +1069,10 @@
     <t>Chưa</t>
   </si>
   <si>
-    <t>Báo cáo thử nghiệm lâm sàng 4 tuần tại Vinmec Times City: 1,500 ca tiếp nhận, 78% containment, tiết kiệm 200 giờ trực điều dưỡng, giảm 35% ca chờ đợi tại Cấp cứu.</t>
-  </si>
-  <si>
-    <t>Ninh Quang Minh &amp; BS. Trưởng khoa Cấp cứu · Deadline: 15/11/2026</t>
+    <t>Báo cáo thử nghiệm 4 tuần tại BV Vinmec Times City: 1.500 ca tiếp nhận, containment 78%, tiết kiệm 200 giờ trực điều dưỡng, giảm 35% ca chờ tại cấp cứu.</t>
+  </si>
+  <si>
+    <t>Ninh Quang Minh và Trưởng khoa Cấp cứu · 15/11/2026</t>
   </si>
   <si>
     <t>Ô nào CHƯA CÓ thì ghi deadline — đừng bỏ trống. Thành thật về khoảng trống được điểm cao hơn bịa nội dung.</t>
@@ -1499,7 +1499,7 @@
     <numFmt numFmtId="169" formatCode="#,##0.0\×"/>
     <numFmt numFmtId="170" formatCode="#,##0&quot; ₫&quot;"/>
   </numFmts>
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1507,42 +1507,9 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="14"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="9"/>
-      <color rgb="FF666666"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF1F2937"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF0000FF"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF008000"/>
-      <name val="Arial"/>
     </font>
     <font>
       <b/>
@@ -1552,15 +1519,12 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <color rgb="FFC00000"/>
-      <name val="Arial"/>
+      <sz val="13"/>
+      <name val="Times New Roman"/>
     </font>
     <font>
-      <b/>
-      <sz val="10"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
+      <sz val="13"/>
+      <name val="Times New Roman"/>
     </font>
   </fonts>
   <fills count="7">
@@ -1633,58 +1597,55 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="43">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+  <cellXfs count="40">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="3" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="9" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="6" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="7" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="9" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="6" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="169" fontId="6" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="9" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="6" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="9" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="9" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="170" fontId="6" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="6" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="4" fontId="9" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="169" fontId="9" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="6" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="4" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="4" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="4" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="4" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="3" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="4" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="4" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="4" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="4" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="3" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="170" fontId="4" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="4" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="169" fontId="4" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="3" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="4" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="3" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="3" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="4" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="4" fontId="3" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="169" fontId="3" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1911,141 +1872,144 @@
     <col min="9" max="26" width="8.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-    </row>
-    <row r="2" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A2" s="3" t="s">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+    </row>
+    <row r="2" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="5" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A4" s="4" t="s">
+    <row r="3" spans="1:8" ht="14.5" x14ac:dyDescent="0.35"/>
+    <row r="4" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="6" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A5" s="5" t="s">
+    <row r="5" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="5" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="5" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="5" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A8" s="11" t="s">
+    <row r="8" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="5" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A10" s="4" t="s">
+    <row r="9" spans="1:8" ht="14.5" x14ac:dyDescent="0.35"/>
+    <row r="10" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="6" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A11" s="12" t="s">
+    <row r="11" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="5" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A12" s="12" t="s">
+    <row r="12" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B12" s="6" t="s">
+      <c r="B12" s="5" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A13" s="12" t="s">
+    <row r="13" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="B13" s="5" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A14" s="12" t="s">
+    <row r="14" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B14" s="6" t="s">
+      <c r="B14" s="5" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A15" s="12" t="s">
+    <row r="15" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="B15" s="5" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A16" s="12" t="s">
+    <row r="16" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="B16" s="6" t="s">
+      <c r="B16" s="5" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="18" spans="1:1" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A18" s="4" t="s">
+    <row r="17" spans="1:1" ht="14.5" x14ac:dyDescent="0.35"/>
+    <row r="18" spans="1:1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="6" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="19" spans="1:1" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A19" s="6" t="s">
+    <row r="19" spans="1:1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="5" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="20" spans="1:1" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A20" s="6" t="s">
+    <row r="20" spans="1:1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="5" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="21" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="6" t="s">
+      <c r="A21" s="5" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="22" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="23" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="3" t="s">
+      <c r="A23" s="5" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="24" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="3" t="s">
+      <c r="A24" s="5" t="s">
         <v>29</v>
       </c>
     </row>
@@ -3043,759 +3007,762 @@
     <col min="9" max="26" width="8.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-    </row>
-    <row r="2" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A2" s="3" t="s">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+    </row>
+    <row r="2" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="5" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A4" s="7" t="s">
+    <row r="3" spans="1:8" ht="14.5" x14ac:dyDescent="0.35"/>
+    <row r="4" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="B4" s="10"/>
-      <c r="C4" s="10"/>
-      <c r="D4" s="10"/>
-      <c r="E4" s="10"/>
-      <c r="F4" s="10"/>
-      <c r="G4" s="10"/>
-      <c r="H4" s="10"/>
-    </row>
-    <row r="5" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A5" s="6" t="s">
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
+    </row>
+    <row r="5" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="5" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A6" s="6" t="s">
+    <row r="6" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="B6" s="13" t="s">
+      <c r="B6" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="5" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A8" s="7" t="s">
+    <row r="7" spans="1:8" ht="14.5" x14ac:dyDescent="0.35"/>
+    <row r="8" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="B8" s="10"/>
-      <c r="C8" s="10"/>
-      <c r="D8" s="10"/>
-      <c r="E8" s="10"/>
-      <c r="F8" s="10"/>
-      <c r="G8" s="10"/>
-      <c r="H8" s="10"/>
-    </row>
-    <row r="9" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A9" s="6" t="s">
+      <c r="B8" s="2"/>
+      <c r="C8" s="2"/>
+      <c r="D8" s="2"/>
+      <c r="E8" s="2"/>
+      <c r="F8" s="2"/>
+      <c r="G8" s="2"/>
+      <c r="H8" s="2"/>
+    </row>
+    <row r="9" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="B9" s="14">
+      <c r="B9" s="13">
         <v>5000</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="5" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A10" s="6" t="s">
+    <row r="10" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="B10" s="15">
+      <c r="B10" s="14">
         <v>0.78</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="D10" s="5" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A11" s="6" t="s">
+    <row r="11" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="B11" s="17">
+      <c r="B11" s="15">
         <f>B9*B10</f>
         <v>3900</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="C11" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="D11" s="5" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A12" s="6" t="s">
+    <row r="12" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="B12" s="17">
+      <c r="B12" s="15">
         <f>B9-B11</f>
         <v>1100</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C12" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="D12" s="5" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A14" s="7" t="s">
+    <row r="13" spans="1:8" ht="14.5" x14ac:dyDescent="0.35"/>
+    <row r="14" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="B14" s="10"/>
-      <c r="C14" s="10"/>
-      <c r="D14" s="10"/>
-      <c r="E14" s="10"/>
-      <c r="F14" s="10"/>
-      <c r="G14" s="10"/>
-      <c r="H14" s="10"/>
-    </row>
-    <row r="15" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A15" s="6" t="s">
+      <c r="B14" s="2"/>
+      <c r="C14" s="2"/>
+      <c r="D14" s="2"/>
+      <c r="E14" s="2"/>
+      <c r="F14" s="2"/>
+      <c r="G14" s="2"/>
+      <c r="H14" s="2"/>
+    </row>
+    <row r="15" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="B15" s="20">
+      <c r="B15" s="16">
         <v>1</v>
       </c>
-      <c r="D15" s="3" t="s">
+      <c r="D15" s="5" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A16" s="6" t="s">
+    <row r="16" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="B16" s="20">
+      <c r="B16" s="16">
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A17" s="6" t="s">
+    <row r="17" spans="1:4" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="B17" s="20">
+      <c r="B17" s="16">
         <v>1.25</v>
       </c>
-      <c r="D17" s="3" t="s">
+      <c r="D17" s="5" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A18" s="6" t="s">
+    <row r="18" spans="1:4" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="B18" s="20">
+      <c r="B18" s="16">
         <v>0.1</v>
       </c>
-      <c r="D18" s="3" t="s">
+      <c r="D18" s="5" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A19" s="6" t="s">
+    <row r="19" spans="1:4" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="B19" s="14">
+      <c r="B19" s="13">
         <v>5</v>
       </c>
-      <c r="C19" s="3" t="s">
+      <c r="C19" s="5" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A20" s="6" t="s">
+    <row r="20" spans="1:4" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="B20" s="14">
+      <c r="B20" s="13">
         <v>3500</v>
       </c>
-      <c r="C20" s="3" t="s">
+      <c r="C20" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="D20" s="3" t="s">
+      <c r="D20" s="5" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="6" t="s">
+      <c r="A21" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="B21" s="14">
+      <c r="B21" s="13">
         <v>800</v>
       </c>
-      <c r="C21" s="3" t="s">
+      <c r="C21" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="D21" s="3" t="s">
+      <c r="D21" s="5" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="6" t="s">
+      <c r="A22" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="B22" s="14">
+      <c r="B22" s="13">
         <v>350</v>
       </c>
-      <c r="C22" s="3" t="s">
+      <c r="C22" s="5" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="6" t="s">
+      <c r="A23" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="B23" s="22">
+      <c r="B23" s="17">
         <f>B20*B17/1000000</f>
         <v>4.3750000000000004E-3</v>
       </c>
     </row>
     <row r="24" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="6" t="s">
+      <c r="A24" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="B24" s="22">
+      <c r="B24" s="17">
         <f>(B19-1)*B20*B18/1000000</f>
         <v>1.4E-3</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="6" t="s">
+      <c r="A25" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="B25" s="22">
+      <c r="B25" s="17">
         <f>B19*B21*B15/1000000</f>
         <v>4.0000000000000001E-3</v>
       </c>
     </row>
     <row r="26" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="6" t="s">
+      <c r="A26" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="B26" s="22">
+      <c r="B26" s="17">
         <f>B19*B22*B16/1000000</f>
         <v>8.7500000000000008E-3</v>
       </c>
     </row>
     <row r="27" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="12" t="s">
+      <c r="A27" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="B27" s="21">
+      <c r="B27" s="18">
         <f>SUM(B23:B26)</f>
         <v>1.8525E-2</v>
       </c>
     </row>
     <row r="28" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="6" t="s">
+      <c r="A28" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="B28" s="22">
+      <c r="B28" s="17">
         <f>B19*(B20+B21)*B15/1000000+B26</f>
         <v>3.0249999999999999E-2</v>
       </c>
     </row>
     <row r="29" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="6" t="s">
+      <c r="A29" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="B29" s="26">
+      <c r="B29" s="19">
         <f>IF(B28=0,0,1-B27/B28)</f>
         <v>0.38760330578512392</v>
       </c>
-      <c r="D29" s="3" t="s">
+      <c r="D29" s="5" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="30" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="6" t="s">
+      <c r="A30" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="B30" s="14">
+      <c r="B30" s="13">
         <v>0</v>
       </c>
-      <c r="D30" s="3" t="s">
+      <c r="D30" s="5" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="31" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="12" t="s">
+      <c r="A31" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="B31" s="21">
+      <c r="B31" s="18">
         <f>B27*(1-B30*0.5)</f>
         <v>1.8525E-2</v>
       </c>
     </row>
     <row r="32" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="33" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A33" s="7" t="s">
+      <c r="A33" s="11" t="s">
         <v>75</v>
       </c>
-      <c r="B33" s="10"/>
-      <c r="C33" s="10"/>
-      <c r="D33" s="10"/>
-      <c r="E33" s="10"/>
-      <c r="F33" s="10"/>
-      <c r="G33" s="10"/>
-      <c r="H33" s="10"/>
+      <c r="B33" s="2"/>
+      <c r="C33" s="2"/>
+      <c r="D33" s="2"/>
+      <c r="E33" s="2"/>
+      <c r="F33" s="2"/>
+      <c r="G33" s="2"/>
+      <c r="H33" s="2"/>
     </row>
     <row r="34" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="6" t="s">
+      <c r="A34" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="B34" s="27">
+      <c r="B34" s="20">
         <v>0</v>
       </c>
-      <c r="D34" s="3" t="s">
+      <c r="D34" s="5" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="35" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="6" t="s">
+      <c r="A35" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="B35" s="19">
+      <c r="B35" s="21">
         <v>0</v>
       </c>
-      <c r="C35" s="3" t="s">
+      <c r="C35" s="5" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="36" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="6" t="s">
+      <c r="A36" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="B36" s="20">
+      <c r="B36" s="16">
         <v>0</v>
       </c>
-      <c r="D36" s="3" t="s">
+      <c r="D36" s="5" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="37" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="6" t="s">
+      <c r="A37" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="B37" s="14">
+      <c r="B37" s="13">
         <v>0</v>
       </c>
-      <c r="C37" s="3" t="s">
+      <c r="C37" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="D37" s="3" t="s">
+      <c r="D37" s="5" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="38" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="6" t="s">
+      <c r="A38" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="B38" s="22">
+      <c r="B38" s="17">
         <f>B34*B35+B36*B37/1000000</f>
         <v>0</v>
       </c>
     </row>
     <row r="39" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="40" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A40" s="7" t="s">
+      <c r="A40" s="11" t="s">
         <v>86</v>
       </c>
-      <c r="B40" s="10"/>
-      <c r="C40" s="10"/>
-      <c r="D40" s="10"/>
-      <c r="E40" s="10"/>
-      <c r="F40" s="10"/>
-      <c r="G40" s="10"/>
-      <c r="H40" s="10"/>
+      <c r="B40" s="2"/>
+      <c r="C40" s="2"/>
+      <c r="D40" s="2"/>
+      <c r="E40" s="2"/>
+      <c r="F40" s="2"/>
+      <c r="G40" s="2"/>
+      <c r="H40" s="2"/>
     </row>
     <row r="41" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A41" s="6" t="s">
+      <c r="A41" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="B41" s="27">
+      <c r="B41" s="20">
         <v>8.0000000000000002E-3</v>
       </c>
-      <c r="D41" s="3" t="s">
+      <c r="D41" s="5" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="42" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A42" s="6" t="s">
+      <c r="A42" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="B42" s="27">
+      <c r="B42" s="20">
         <v>0</v>
       </c>
     </row>
     <row r="43" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A43" s="6" t="s">
+      <c r="A43" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="B43" s="22">
+      <c r="B43" s="17">
         <f>B41+B42*B35</f>
         <v>8.0000000000000002E-3</v>
       </c>
     </row>
     <row r="44" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="45" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A45" s="7" t="s">
+      <c r="A45" s="11" t="s">
         <v>91</v>
       </c>
-      <c r="B45" s="10"/>
-      <c r="C45" s="10"/>
-      <c r="D45" s="10"/>
-      <c r="E45" s="10"/>
-      <c r="F45" s="10"/>
-      <c r="G45" s="10"/>
-      <c r="H45" s="10"/>
+      <c r="B45" s="2"/>
+      <c r="C45" s="2"/>
+      <c r="D45" s="2"/>
+      <c r="E45" s="2"/>
+      <c r="F45" s="2"/>
+      <c r="G45" s="2"/>
+      <c r="H45" s="2"/>
     </row>
     <row r="46" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A46" s="6" t="s">
+      <c r="A46" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="B46" s="15">
+      <c r="B46" s="14">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="D46" s="3" t="s">
+      <c r="D46" s="5" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="47" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A47" s="6" t="s">
+      <c r="A47" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="B47" s="22">
+      <c r="B47" s="17">
         <f>(B31+B38)*B46</f>
         <v>1.2967500000000002E-3</v>
       </c>
     </row>
     <row r="48" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="49" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A49" s="7" t="s">
+      <c r="A49" s="11" t="s">
         <v>95</v>
       </c>
-      <c r="B49" s="10"/>
-      <c r="C49" s="10"/>
-      <c r="D49" s="10"/>
-      <c r="E49" s="10"/>
-      <c r="F49" s="10"/>
-      <c r="G49" s="10"/>
-      <c r="H49" s="10"/>
+      <c r="B49" s="2"/>
+      <c r="C49" s="2"/>
+      <c r="D49" s="2"/>
+      <c r="E49" s="2"/>
+      <c r="F49" s="2"/>
+      <c r="G49" s="2"/>
+      <c r="H49" s="2"/>
     </row>
     <row r="50" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A50" s="6" t="s">
+      <c r="A50" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="B50" s="20">
+      <c r="B50" s="16">
         <v>7</v>
       </c>
-      <c r="D50" s="3" t="s">
+      <c r="D50" s="5" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="51" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A51" s="6" t="s">
+      <c r="A51" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="B51" s="15">
+      <c r="B51" s="14">
         <v>0.06</v>
       </c>
-      <c r="D51" s="3" t="s">
+      <c r="D51" s="5" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="52" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A52" s="6" t="s">
+      <c r="A52" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="B52" s="19">
+      <c r="B52" s="21">
         <v>3</v>
       </c>
-      <c r="C52" s="3" t="s">
+      <c r="C52" s="5" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="53" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A53" s="6" t="s">
+      <c r="A53" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="B53" s="19">
+      <c r="B53" s="21">
         <v>5</v>
       </c>
-      <c r="C53" s="3" t="s">
+      <c r="C53" s="5" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="54" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A54" s="6" t="s">
+      <c r="A54" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="B54" s="30">
+      <c r="B54" s="22">
         <f>B9*B51*(B52/60)*B50</f>
         <v>105</v>
       </c>
     </row>
     <row r="55" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A55" s="6" t="s">
+      <c r="A55" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="B55" s="30">
+      <c r="B55" s="22">
         <f>IF(B6="B",B12*(B53/60)*B50,0)</f>
         <v>641.66666666666663</v>
       </c>
-      <c r="D55" s="3" t="s">
+      <c r="D55" s="5" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="56" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A56" s="12" t="s">
+      <c r="A56" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="B56" s="31">
+      <c r="B56" s="23">
         <f>B54+B55</f>
         <v>746.66666666666663</v>
       </c>
     </row>
     <row r="57" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="58" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A58" s="7" t="s">
+      <c r="A58" s="11" t="s">
         <v>106</v>
       </c>
-      <c r="B58" s="10"/>
-      <c r="C58" s="10"/>
-      <c r="D58" s="10"/>
-      <c r="E58" s="10"/>
-      <c r="F58" s="10"/>
-      <c r="G58" s="10"/>
-      <c r="H58" s="10"/>
+      <c r="B58" s="2"/>
+      <c r="C58" s="2"/>
+      <c r="D58" s="2"/>
+      <c r="E58" s="2"/>
+      <c r="F58" s="2"/>
+      <c r="G58" s="2"/>
+      <c r="H58" s="2"/>
     </row>
     <row r="59" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A59" s="6" t="s">
+      <c r="A59" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="B59" s="20">
+      <c r="B59" s="16">
         <v>0</v>
       </c>
-      <c r="D59" s="3" t="s">
+      <c r="D59" s="5" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="60" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="61" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A61" s="7" t="s">
+      <c r="A61" s="11" t="s">
         <v>109</v>
       </c>
-      <c r="B61" s="10"/>
-      <c r="C61" s="10"/>
-      <c r="D61" s="10"/>
-      <c r="E61" s="10"/>
-      <c r="F61" s="10"/>
-      <c r="G61" s="10"/>
-      <c r="H61" s="10"/>
+      <c r="B61" s="2"/>
+      <c r="C61" s="2"/>
+      <c r="D61" s="2"/>
+      <c r="E61" s="2"/>
+      <c r="F61" s="2"/>
+      <c r="G61" s="2"/>
+      <c r="H61" s="2"/>
     </row>
     <row r="62" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A62" s="6" t="s">
+      <c r="A62" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="B62" s="30">
+      <c r="B62" s="22">
         <f>B9*(B31+B38+B43+B47)</f>
         <v>139.10874999999999</v>
       </c>
     </row>
     <row r="63" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A63" s="6" t="s">
+      <c r="A63" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="B63" s="30">
+      <c r="B63" s="22">
         <f>B56</f>
         <v>746.66666666666663</v>
       </c>
     </row>
     <row r="64" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A64" s="6" t="s">
+      <c r="A64" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="B64" s="30">
+      <c r="B64" s="22">
         <f>B59</f>
         <v>0</v>
       </c>
     </row>
     <row r="65" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A65" s="6" t="s">
+      <c r="A65" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="B65" s="30">
+      <c r="B65" s="22">
         <f>B62+B63+B64</f>
         <v>885.77541666666662</v>
       </c>
     </row>
     <row r="66" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A66" s="12" t="s">
+      <c r="A66" s="6" t="s">
         <v>114</v>
       </c>
-      <c r="B66" s="21">
+      <c r="B66" s="18">
         <f>IF(B11=0,0,(B62+B63)/B11)</f>
         <v>0.22712190170940169</v>
       </c>
-      <c r="C66" s="3" t="s">
+      <c r="C66" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="D66" s="3" t="s">
+      <c r="D66" s="5" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="67" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A67" s="12" t="s">
+      <c r="A67" s="6" t="s">
         <v>117</v>
       </c>
-      <c r="B67" s="21">
+      <c r="B67" s="18">
         <f>IF(B11=0,0,B65/B11)</f>
         <v>0.22712190170940169</v>
       </c>
-      <c r="C67" s="3" t="s">
+      <c r="C67" s="5" t="s">
         <v>115</v>
       </c>
     </row>
     <row r="68" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A68" s="6" t="s">
+      <c r="A68" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="B68" s="14">
+      <c r="B68" s="13">
         <v>26000</v>
       </c>
-      <c r="C68" s="3" t="s">
+      <c r="C68" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="D68" s="3" t="s">
+      <c r="D68" s="5" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="69" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A69" s="6" t="s">
+      <c r="A69" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="B69" s="34">
+      <c r="B69" s="24">
         <f>B66*B68</f>
         <v>5905.1694444444438</v>
       </c>
-      <c r="C69" s="3" t="s">
+      <c r="C69" s="5" t="s">
         <v>122</v>
       </c>
     </row>
     <row r="70" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="71" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A71" s="7" t="s">
+      <c r="A71" s="11" t="s">
         <v>123</v>
       </c>
-      <c r="B71" s="10"/>
-      <c r="C71" s="10"/>
-      <c r="D71" s="10"/>
-      <c r="E71" s="10"/>
-      <c r="F71" s="10"/>
-      <c r="G71" s="10"/>
-      <c r="H71" s="10"/>
+      <c r="B71" s="2"/>
+      <c r="C71" s="2"/>
+      <c r="D71" s="2"/>
+      <c r="E71" s="2"/>
+      <c r="F71" s="2"/>
+      <c r="G71" s="2"/>
+      <c r="H71" s="2"/>
     </row>
     <row r="72" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A72" s="6" t="s">
+      <c r="A72" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="B72" s="30">
+      <c r="B72" s="22">
         <f>B9*B31</f>
         <v>92.625</v>
       </c>
-      <c r="C72" s="26">
+      <c r="C72" s="19">
         <f t="shared" ref="C72:C77" si="0">IF($B$65=0,0,B72/$B$65)</f>
         <v>0.10456939564722248</v>
       </c>
     </row>
     <row r="73" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A73" s="6" t="s">
+      <c r="A73" s="5" t="s">
         <v>125</v>
       </c>
-      <c r="B73" s="30">
+      <c r="B73" s="22">
         <f>B9*B38</f>
         <v>0</v>
       </c>
-      <c r="C73" s="26">
+      <c r="C73" s="19">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="74" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A74" s="6" t="s">
+      <c r="A74" s="5" t="s">
         <v>126</v>
       </c>
-      <c r="B74" s="30">
+      <c r="B74" s="22">
         <f>B9*B43</f>
         <v>40</v>
       </c>
-      <c r="C74" s="26">
+      <c r="C74" s="19">
         <f t="shared" si="0"/>
         <v>4.5158173558854507E-2</v>
       </c>
     </row>
     <row r="75" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A75" s="6" t="s">
+      <c r="A75" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="B75" s="30">
+      <c r="B75" s="22">
         <f>B9*B47</f>
         <v>6.4837500000000006</v>
       </c>
-      <c r="C75" s="26">
+      <c r="C75" s="19">
         <f t="shared" si="0"/>
         <v>7.3198576953055735E-3</v>
       </c>
     </row>
     <row r="76" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A76" s="6" t="s">
+      <c r="A76" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="B76" s="30">
+      <c r="B76" s="22">
         <f>B56</f>
         <v>746.66666666666663</v>
       </c>
-      <c r="C76" s="26">
+      <c r="C76" s="19">
         <f t="shared" si="0"/>
         <v>0.84295257309861749</v>
       </c>
     </row>
     <row r="77" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A77" s="6" t="s">
+      <c r="A77" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="B77" s="30">
+      <c r="B77" s="22">
         <f>B59</f>
         <v>0</v>
       </c>
-      <c r="C77" s="26">
+      <c r="C77" s="19">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="78" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A78" s="3" t="s">
+      <c r="A78" s="5" t="s">
         <v>130</v>
       </c>
     </row>
@@ -4745,212 +4712,215 @@
     <col min="9" max="26" width="8.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-    </row>
-    <row r="2" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A2" s="3" t="s">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+    </row>
+    <row r="2" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="5" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A4" s="7" t="s">
+    <row r="3" spans="1:8" ht="14.5" x14ac:dyDescent="0.35"/>
+    <row r="4" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="11" t="s">
         <v>133</v>
       </c>
-      <c r="B4" s="10"/>
-      <c r="C4" s="10"/>
-      <c r="D4" s="10"/>
-      <c r="E4" s="10"/>
-      <c r="F4" s="10"/>
-      <c r="G4" s="10"/>
-      <c r="H4" s="10"/>
-    </row>
-    <row r="5" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A5" s="6" t="s">
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
+    </row>
+    <row r="5" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="5" t="s">
         <v>134</v>
       </c>
-      <c r="B5" s="18">
+      <c r="B5" s="17">
         <f>'1_Cost_Job'!B66</f>
         <v>0.22712190170940169</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="5" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A6" s="6" t="s">
+    <row r="6" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="B6" s="19">
+      <c r="B6" s="21">
         <v>3</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="5" t="s">
         <v>136</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="5" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A7" s="12" t="s">
+    <row r="7" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="6" t="s">
         <v>138</v>
       </c>
-      <c r="B7" s="21">
+      <c r="B7" s="18">
         <f>B5*B6</f>
         <v>0.68136570512820505</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="5" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A9" s="7" t="s">
+    <row r="8" spans="1:8" ht="14.5" x14ac:dyDescent="0.35"/>
+    <row r="9" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="11" t="s">
         <v>139</v>
       </c>
-      <c r="B9" s="10"/>
-      <c r="C9" s="10"/>
-      <c r="D9" s="10"/>
-      <c r="E9" s="10"/>
-      <c r="F9" s="10"/>
-      <c r="G9" s="10"/>
-      <c r="H9" s="10"/>
-    </row>
-    <row r="10" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A10" s="6" t="s">
+      <c r="B9" s="2"/>
+      <c r="C9" s="2"/>
+      <c r="D9" s="2"/>
+      <c r="E9" s="2"/>
+      <c r="F9" s="2"/>
+      <c r="G9" s="2"/>
+      <c r="H9" s="2"/>
+    </row>
+    <row r="10" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="B10" s="23">
+      <c r="B10" s="25">
         <v>4500</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="D10" s="5" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A11" s="6" t="s">
+    <row r="11" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="5" t="s">
         <v>142</v>
       </c>
-      <c r="B11" s="14">
+      <c r="B11" s="13">
         <v>1000</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="C11" s="5" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A12" s="6" t="s">
+    <row r="12" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="B12" s="22">
+      <c r="B12" s="17">
         <f>IF(B11=0,0,B10*0.1/B11)</f>
         <v>0.45</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C12" s="5" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A13" s="6" t="s">
+    <row r="13" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="B13" s="22">
+      <c r="B13" s="17">
         <f>IF(B11=0,0,B10*0.25/B11)</f>
         <v>1.125</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C13" s="5" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A14" s="6" t="s">
+    <row r="14" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="B14" s="23">
+      <c r="B14" s="25">
         <v>1200</v>
       </c>
-      <c r="D14" s="3" t="s">
+      <c r="D14" s="5" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A15" s="6" t="s">
+    <row r="15" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="5" t="s">
         <v>147</v>
       </c>
-      <c r="B15" s="22">
+      <c r="B15" s="17">
         <f>IF(B11=0,0,B14*0.5/B11)</f>
         <v>0.6</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="C15" s="5" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A16" s="6" t="s">
+    <row r="16" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="5" t="s">
         <v>148</v>
       </c>
-      <c r="B16" s="22">
+      <c r="B16" s="17">
         <f>IF(B11=0,0,B14*0.7/B11)</f>
         <v>0.84</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C16" s="5" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A18" s="7" t="s">
+    <row r="17" spans="1:8" ht="14.5" x14ac:dyDescent="0.35"/>
+    <row r="18" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="11" t="s">
         <v>149</v>
       </c>
-      <c r="B18" s="10"/>
-      <c r="C18" s="10"/>
-      <c r="D18" s="10"/>
-      <c r="E18" s="10"/>
-      <c r="F18" s="10"/>
-      <c r="G18" s="10"/>
-      <c r="H18" s="10"/>
-    </row>
-    <row r="19" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A19" s="6" t="s">
+      <c r="B18" s="2"/>
+      <c r="C18" s="2"/>
+      <c r="D18" s="2"/>
+      <c r="E18" s="2"/>
+      <c r="F18" s="2"/>
+      <c r="G18" s="2"/>
+      <c r="H18" s="2"/>
+    </row>
+    <row r="19" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="B19" s="27">
+      <c r="B19" s="20">
         <v>0.79</v>
       </c>
-      <c r="C19" s="3" t="s">
+      <c r="C19" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="D19" s="3" t="s">
+      <c r="D19" s="5" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A20" s="6" t="s">
+    <row r="20" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="B20" s="28">
+      <c r="B20" s="26">
         <f>IF(B5=0,0,B19/B5)</f>
         <v>3.4783083183707686</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="12" t="s">
+      <c r="A21" s="6" t="s">
         <v>153</v>
       </c>
-      <c r="B21" s="29">
+      <c r="B21" s="27">
         <f>IF(B19=0,0,(B19-B5)/B19)</f>
         <v>0.71250392188683331</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="6" t="s">
+      <c r="A22" s="5" t="s">
         <v>154</v>
       </c>
       <c r="B22" s="8" t="str">
@@ -4959,7 +4929,7 @@
       </c>
     </row>
     <row r="23" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="6" t="s">
+      <c r="A23" s="5" t="s">
         <v>155</v>
       </c>
       <c r="B23" s="8" t="str">
@@ -4968,7 +4938,7 @@
       </c>
     </row>
     <row r="24" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="6" t="s">
+      <c r="A24" s="5" t="s">
         <v>156</v>
       </c>
       <c r="B24" s="8" t="str">
@@ -4977,7 +4947,7 @@
       </c>
     </row>
     <row r="25" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="6" t="s">
+      <c r="A25" s="5" t="s">
         <v>157</v>
       </c>
       <c r="B25" s="8" t="str">
@@ -4987,80 +4957,80 @@
     </row>
     <row r="26" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="27" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="7" t="s">
+      <c r="A27" s="11" t="s">
         <v>158</v>
       </c>
-      <c r="B27" s="10"/>
-      <c r="C27" s="10"/>
-      <c r="D27" s="10"/>
-      <c r="E27" s="10"/>
-      <c r="F27" s="10"/>
-      <c r="G27" s="10"/>
-      <c r="H27" s="10"/>
+      <c r="B27" s="2"/>
+      <c r="C27" s="2"/>
+      <c r="D27" s="2"/>
+      <c r="E27" s="2"/>
+      <c r="F27" s="2"/>
+      <c r="G27" s="2"/>
+      <c r="H27" s="2"/>
     </row>
     <row r="28" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="3" t="s">
+      <c r="A28" s="5" t="s">
         <v>159</v>
       </c>
     </row>
     <row r="29" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="6" t="s">
+      <c r="A29" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="B29" s="18">
+      <c r="B29" s="17">
         <f>'1_Cost_Job'!B31+'1_Cost_Job'!B38+'1_Cost_Job'!B43+'1_Cost_Job'!B47</f>
         <v>2.7821749999999999E-2</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="6" t="s">
+      <c r="A30" s="5" t="s">
         <v>161</v>
       </c>
-      <c r="B30" s="18">
+      <c r="B30" s="17">
         <f>'1_Cost_Job'!B51*('1_Cost_Job'!B52/60)*'1_Cost_Job'!B50</f>
         <v>2.1000000000000001E-2</v>
       </c>
     </row>
     <row r="31" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="6" t="s">
+      <c r="A31" s="5" t="s">
         <v>162</v>
       </c>
-      <c r="B31" s="18">
+      <c r="B31" s="17">
         <f>IF('1_Cost_Job'!B6="B",('1_Cost_Job'!B53/60)*'1_Cost_Job'!B50,0)</f>
         <v>0.58333333333333326</v>
       </c>
     </row>
     <row r="32" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="6" t="s">
+      <c r="A32" s="5" t="s">
         <v>163</v>
       </c>
-      <c r="B32" s="15">
+      <c r="B32" s="14">
         <v>0.6</v>
       </c>
     </row>
     <row r="33" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A33" s="12" t="s">
+      <c r="A33" s="6" t="s">
         <v>164</v>
       </c>
-      <c r="B33" s="29">
+      <c r="B33" s="27">
         <f>IF((B19*(1-B32)+B31)=0,0,(B29+B30+B31)/(B19*(1-B32)+B31))</f>
         <v>0.70291521497405474</v>
       </c>
-      <c r="D33" s="3" t="s">
+      <c r="D33" s="5" t="s">
         <v>165</v>
       </c>
     </row>
     <row r="34" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="6" t="s">
+      <c r="A34" s="5" t="s">
         <v>166</v>
       </c>
-      <c r="B34" s="32">
+      <c r="B34" s="19">
         <f>'1_Cost_Job'!B10</f>
         <v>0.78</v>
       </c>
     </row>
     <row r="35" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="6" t="s">
+      <c r="A35" s="5" t="s">
         <v>167</v>
       </c>
       <c r="B35" s="8" t="str">
@@ -5070,40 +5040,40 @@
     </row>
     <row r="36" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="37" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="7" t="s">
+      <c r="A37" s="11" t="s">
         <v>168</v>
       </c>
-      <c r="B37" s="10"/>
-      <c r="C37" s="10"/>
-      <c r="D37" s="10"/>
-      <c r="E37" s="10"/>
-      <c r="F37" s="10"/>
-      <c r="G37" s="10"/>
-      <c r="H37" s="10"/>
+      <c r="B37" s="2"/>
+      <c r="C37" s="2"/>
+      <c r="D37" s="2"/>
+      <c r="E37" s="2"/>
+      <c r="F37" s="2"/>
+      <c r="G37" s="2"/>
+      <c r="H37" s="2"/>
     </row>
     <row r="38" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="25" t="s">
+      <c r="A38" s="28" t="s">
         <v>169</v>
       </c>
-      <c r="B38" s="25" t="s">
+      <c r="B38" s="28" t="s">
         <v>170</v>
       </c>
-      <c r="C38" s="25" t="s">
+      <c r="C38" s="28" t="s">
         <v>171</v>
       </c>
-      <c r="D38" s="25" t="s">
+      <c r="D38" s="28" t="s">
         <v>172</v>
       </c>
     </row>
     <row r="39" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="38">
+      <c r="A39" s="29">
         <v>0.5</v>
       </c>
-      <c r="B39" s="22">
+      <c r="B39" s="17">
         <f t="shared" ref="B39:B44" si="0">($B$29+$B$30+$B$31*(1-A39))/A39</f>
         <v>0.68097683333333325</v>
       </c>
-      <c r="C39" s="26">
+      <c r="C39" s="19">
         <f t="shared" ref="C39:C44" si="1">IF($B$19=0,0,1-B39/$B$19)</f>
         <v>0.13800400843881866</v>
       </c>
@@ -5113,14 +5083,14 @@
       </c>
     </row>
     <row r="40" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A40" s="38">
+      <c r="A40" s="29">
         <v>0.6</v>
       </c>
-      <c r="B40" s="22">
+      <c r="B40" s="17">
         <f t="shared" si="0"/>
         <v>0.47025847222222217</v>
       </c>
-      <c r="C40" s="26">
+      <c r="C40" s="19">
         <f t="shared" si="1"/>
         <v>0.40473611111111119</v>
       </c>
@@ -5130,14 +5100,14 @@
       </c>
     </row>
     <row r="41" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A41" s="38">
+      <c r="A41" s="29">
         <v>0.7</v>
       </c>
-      <c r="B41" s="22">
+      <c r="B41" s="17">
         <f t="shared" si="0"/>
         <v>0.31974535714285718</v>
       </c>
-      <c r="C41" s="26">
+      <c r="C41" s="19">
         <f t="shared" si="1"/>
         <v>0.59525904159132004</v>
       </c>
@@ -5147,14 +5117,14 @@
       </c>
     </row>
     <row r="42" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A42" s="38">
+      <c r="A42" s="29">
         <v>0.8</v>
       </c>
-      <c r="B42" s="22">
+      <c r="B42" s="17">
         <f t="shared" si="0"/>
         <v>0.20686052083333328</v>
       </c>
-      <c r="C42" s="26">
+      <c r="C42" s="19">
         <f t="shared" si="1"/>
         <v>0.73815123945147687</v>
       </c>
@@ -5164,14 +5134,14 @@
       </c>
     </row>
     <row r="43" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A43" s="38">
+      <c r="A43" s="29">
         <v>0.9</v>
       </c>
-      <c r="B43" s="22">
+      <c r="B43" s="17">
         <f t="shared" si="0"/>
         <v>0.11906120370370368</v>
       </c>
-      <c r="C43" s="26">
+      <c r="C43" s="19">
         <f t="shared" si="1"/>
         <v>0.8492896155649321</v>
       </c>
@@ -5181,14 +5151,14 @@
       </c>
     </row>
     <row r="44" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="38">
+      <c r="A44" s="29">
         <v>0.95</v>
       </c>
-      <c r="B44" s="22">
+      <c r="B44" s="17">
         <f t="shared" si="0"/>
         <v>8.2093070175438626E-2</v>
       </c>
-      <c r="C44" s="26">
+      <c r="C44" s="19">
         <f t="shared" si="1"/>
         <v>0.89608472129691319</v>
       </c>
@@ -5199,64 +5169,64 @@
     </row>
     <row r="45" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="46" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A46" s="3" t="s">
+      <c r="A46" s="5" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="47" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="48" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A48" s="7" t="s">
+      <c r="A48" s="11" t="s">
         <v>174</v>
       </c>
-      <c r="B48" s="10"/>
-      <c r="C48" s="10"/>
-      <c r="D48" s="10"/>
-      <c r="E48" s="10"/>
-      <c r="F48" s="10"/>
-      <c r="G48" s="10"/>
-      <c r="H48" s="10"/>
+      <c r="B48" s="2"/>
+      <c r="C48" s="2"/>
+      <c r="D48" s="2"/>
+      <c r="E48" s="2"/>
+      <c r="F48" s="2"/>
+      <c r="G48" s="2"/>
+      <c r="H48" s="2"/>
     </row>
     <row r="49" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A49" s="12" t="s">
+      <c r="A49" s="6" t="s">
         <v>170</v>
       </c>
-      <c r="B49" s="21">
+      <c r="B49" s="18">
         <f>B5</f>
         <v>0.22712190170940169</v>
       </c>
     </row>
     <row r="50" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A50" s="12" t="s">
+      <c r="A50" s="6" t="s">
         <v>175</v>
       </c>
-      <c r="B50" s="21">
+      <c r="B50" s="18">
         <f>B7</f>
         <v>0.68136570512820505</v>
       </c>
     </row>
     <row r="51" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A51" s="12" t="s">
+      <c r="A51" s="6" t="s">
         <v>176</v>
       </c>
-      <c r="B51" s="21">
+      <c r="B51" s="18">
         <f>B19</f>
         <v>0.79</v>
       </c>
     </row>
     <row r="52" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A52" s="12" t="s">
+      <c r="A52" s="6" t="s">
         <v>171</v>
       </c>
-      <c r="B52" s="29">
+      <c r="B52" s="27">
         <f>B21</f>
         <v>0.71250392188683331</v>
       </c>
     </row>
     <row r="53" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A53" s="12" t="s">
+      <c r="A53" s="6" t="s">
         <v>177</v>
       </c>
-      <c r="B53" s="29">
+      <c r="B53" s="27">
         <f>B33</f>
         <v>0.70291521497405474</v>
       </c>
@@ -6227,276 +6197,279 @@
     <col min="9" max="26" width="8.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="4" t="s">
         <v>178</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-    </row>
-    <row r="2" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A2" s="3" t="s">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+    </row>
+    <row r="2" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="5" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A4" s="7" t="s">
+    <row r="3" spans="1:8" ht="14.5" x14ac:dyDescent="0.35"/>
+    <row r="4" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="11" t="s">
         <v>180</v>
       </c>
-      <c r="B4" s="10"/>
-      <c r="C4" s="10"/>
-      <c r="D4" s="10"/>
-      <c r="E4" s="10"/>
-      <c r="F4" s="10"/>
-      <c r="G4" s="10"/>
-      <c r="H4" s="10"/>
-    </row>
-    <row r="5" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A5" s="6" t="s">
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
+    </row>
+    <row r="5" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="5" t="s">
         <v>181</v>
       </c>
-      <c r="B5" s="13">
+      <c r="B5" s="12">
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A6" s="6" t="s">
+    <row r="6" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="5" t="s">
         <v>182</v>
       </c>
-      <c r="B6" s="13">
+      <c r="B6" s="12">
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A7" s="6" t="s">
+    <row r="7" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="5" t="s">
         <v>183</v>
       </c>
-      <c r="B7" s="13">
+      <c r="B7" s="12">
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A8" s="6" t="s">
+    <row r="8" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="5" t="s">
         <v>184</v>
       </c>
-      <c r="B8" s="13">
+      <c r="B8" s="12">
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A9" s="6" t="s">
+    <row r="9" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="5" t="s">
         <v>185</v>
       </c>
-      <c r="B9" s="13">
+      <c r="B9" s="12">
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A10" s="12" t="s">
+    <row r="10" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="6" t="s">
         <v>186</v>
       </c>
-      <c r="B10" s="16">
+      <c r="B10" s="30">
         <f>SUM(B5:B9)</f>
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A12" s="7" t="s">
+    <row r="11" spans="1:8" ht="14.5" x14ac:dyDescent="0.35"/>
+    <row r="12" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="11" t="s">
         <v>187</v>
       </c>
-      <c r="B12" s="10"/>
-      <c r="C12" s="10"/>
-      <c r="D12" s="10"/>
-      <c r="E12" s="10"/>
-      <c r="F12" s="10"/>
-      <c r="G12" s="10"/>
-      <c r="H12" s="10"/>
-    </row>
-    <row r="13" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A13" s="6" t="s">
+      <c r="B12" s="2"/>
+      <c r="C12" s="2"/>
+      <c r="D12" s="2"/>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
+      <c r="G12" s="2"/>
+      <c r="H12" s="2"/>
+    </row>
+    <row r="13" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="5" t="s">
         <v>188</v>
       </c>
-      <c r="B13" s="13">
+      <c r="B13" s="12">
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A14" s="6" t="s">
+    <row r="14" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="5" t="s">
         <v>189</v>
       </c>
-      <c r="B14" s="13">
+      <c r="B14" s="12">
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A15" s="6" t="s">
+    <row r="15" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="5" t="s">
         <v>190</v>
       </c>
-      <c r="B15" s="13">
+      <c r="B15" s="12">
         <v>2</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A16" s="6" t="s">
+    <row r="16" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="5" t="s">
         <v>191</v>
       </c>
-      <c r="B16" s="13">
+      <c r="B16" s="12">
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A17" s="6" t="s">
+    <row r="17" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="5" t="s">
         <v>192</v>
       </c>
-      <c r="B17" s="13">
+      <c r="B17" s="12">
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A18" s="12" t="s">
+    <row r="18" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="6" t="s">
         <v>193</v>
       </c>
-      <c r="B18" s="16">
+      <c r="B18" s="30">
         <f>SUM(B13:B17)</f>
         <v>6</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A20" s="7" t="s">
+    <row r="19" spans="1:8" ht="14.5" x14ac:dyDescent="0.35"/>
+    <row r="20" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="11" t="s">
         <v>194</v>
       </c>
-      <c r="B20" s="10"/>
-      <c r="C20" s="10"/>
-      <c r="D20" s="10"/>
-      <c r="E20" s="10"/>
-      <c r="F20" s="10"/>
-      <c r="G20" s="10"/>
-      <c r="H20" s="10"/>
+      <c r="B20" s="2"/>
+      <c r="C20" s="2"/>
+      <c r="D20" s="2"/>
+      <c r="E20" s="2"/>
+      <c r="F20" s="2"/>
+      <c r="G20" s="2"/>
+      <c r="H20" s="2"/>
     </row>
     <row r="21" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="12" t="s">
+      <c r="A21" s="6" t="s">
         <v>195</v>
       </c>
-      <c r="B21" s="24" t="str">
+      <c r="B21" s="31" t="str">
         <f>IF(AND(B10&gt;=7,B18&gt;=7),"OUTCOME",IF(AND(B10&gt;=7,B18&lt;7),"USAGE",IF(AND(B10&lt;7,B18&gt;=7),"USAGE (an toàn)","SEAT hoặc HYBRID")))</f>
         <v>USAGE</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="3" t="s">
+      <c r="A22" s="5" t="s">
         <v>196</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="24" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="7" t="s">
+      <c r="A24" s="11" t="s">
         <v>197</v>
       </c>
-      <c r="B24" s="10"/>
-      <c r="C24" s="10"/>
-      <c r="D24" s="10"/>
-      <c r="E24" s="10"/>
-      <c r="F24" s="10"/>
-      <c r="G24" s="10"/>
-      <c r="H24" s="10"/>
+      <c r="B24" s="2"/>
+      <c r="C24" s="2"/>
+      <c r="D24" s="2"/>
+      <c r="E24" s="2"/>
+      <c r="F24" s="2"/>
+      <c r="G24" s="2"/>
+      <c r="H24" s="2"/>
     </row>
     <row r="25" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="25" t="s">
+      <c r="A25" s="28" t="s">
         <v>198</v>
       </c>
-      <c r="B25" s="25" t="s">
+      <c r="B25" s="28" t="s">
         <v>199</v>
       </c>
-      <c r="C25" s="25" t="s">
+      <c r="C25" s="28" t="s">
         <v>200</v>
       </c>
-      <c r="D25" s="25" t="s">
+      <c r="D25" s="28" t="s">
         <v>201</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="5" t="s">
+      <c r="A26" s="7" t="s">
         <v>202</v>
       </c>
-      <c r="B26" s="5" t="s">
+      <c r="B26" s="7" t="s">
         <v>203</v>
       </c>
-      <c r="C26" s="5" t="s">
+      <c r="C26" s="7" t="s">
         <v>204</v>
       </c>
-      <c r="D26" s="5" t="s">
+      <c r="D26" s="7" t="s">
         <v>205</v>
       </c>
     </row>
     <row r="27" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="5" t="s">
+      <c r="A27" s="7" t="s">
         <v>206</v>
       </c>
-      <c r="B27" s="5" t="s">
+      <c r="B27" s="7" t="s">
         <v>207</v>
       </c>
-      <c r="C27" s="5" t="s">
+      <c r="C27" s="7" t="s">
         <v>208</v>
       </c>
-      <c r="D27" s="5" t="s">
+      <c r="D27" s="7" t="s">
         <v>209</v>
       </c>
     </row>
     <row r="28" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="29" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="7" t="s">
+      <c r="A29" s="11" t="s">
         <v>210</v>
       </c>
-      <c r="B29" s="10"/>
-      <c r="C29" s="10"/>
-      <c r="D29" s="10"/>
-      <c r="E29" s="10"/>
-      <c r="F29" s="10"/>
-      <c r="G29" s="10"/>
-      <c r="H29" s="10"/>
+      <c r="B29" s="2"/>
+      <c r="C29" s="2"/>
+      <c r="D29" s="2"/>
+      <c r="E29" s="2"/>
+      <c r="F29" s="2"/>
+      <c r="G29" s="2"/>
+      <c r="H29" s="2"/>
     </row>
     <row r="30" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="6" t="s">
+      <c r="A30" s="5" t="s">
         <v>211</v>
       </c>
-      <c r="B30" s="5" t="s">
+      <c r="B30" s="7" t="s">
         <v>212</v>
       </c>
     </row>
     <row r="31" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="6" t="s">
+      <c r="A31" s="5" t="s">
         <v>213</v>
       </c>
-      <c r="B31" s="5" t="s">
+      <c r="B31" s="7" t="s">
         <v>214</v>
       </c>
     </row>
     <row r="32" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="6" t="s">
+      <c r="A32" s="5" t="s">
         <v>215</v>
       </c>
-      <c r="B32" s="5" t="s">
+      <c r="B32" s="7" t="s">
         <v>216</v>
       </c>
     </row>
     <row r="33" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A33" s="6" t="s">
+      <c r="A33" s="5" t="s">
         <v>217</v>
       </c>
-      <c r="B33" s="5" t="s">
+      <c r="B33" s="7" t="s">
         <v>218</v>
       </c>
     </row>
     <row r="34" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="6" t="s">
+      <c r="A34" s="5" t="s">
         <v>219</v>
       </c>
-      <c r="B34" s="5" t="s">
+      <c r="B34" s="7" t="s">
         <v>220</v>
       </c>
     </row>
@@ -7484,153 +7457,155 @@
     <col min="9" max="26" width="8.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="4" t="s">
         <v>221</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-    </row>
-    <row r="2" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A2" s="3" t="s">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+    </row>
+    <row r="2" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="5" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A4" s="7" t="s">
+    <row r="3" spans="1:8" ht="14.5" x14ac:dyDescent="0.35"/>
+    <row r="4" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="11" t="s">
         <v>223</v>
       </c>
-      <c r="B4" s="10"/>
-      <c r="C4" s="10"/>
-      <c r="D4" s="10"/>
-      <c r="E4" s="10"/>
-      <c r="F4" s="10"/>
-      <c r="G4" s="10"/>
-      <c r="H4" s="10"/>
-    </row>
-    <row r="5" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A5" s="6" t="s">
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
+    </row>
+    <row r="5" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="5" t="s">
         <v>224</v>
       </c>
-      <c r="B5" s="23">
+      <c r="B5" s="25">
         <v>790</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A6" s="6" t="s">
+    <row r="6" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="5" t="s">
         <v>225</v>
       </c>
-      <c r="B6" s="32">
+      <c r="B6" s="19">
         <f>'2_Pricing'!B21</f>
         <v>0.71250392188683331</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A7" s="6" t="s">
+    <row r="7" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="5" t="s">
         <v>226</v>
       </c>
-      <c r="B7" s="13" t="s">
+      <c r="B7" s="12" t="s">
         <v>227</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A8" s="6" t="s">
+    <row r="8" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="5" t="s">
         <v>228</v>
       </c>
-      <c r="B8" s="17">
+      <c r="B8" s="15">
         <f>IF(B7="SMB",12,IF(B7="Mid",18,24))</f>
         <v>18</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="5" t="s">
         <v>229</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="5" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A9" s="12" t="s">
+    <row r="9" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="6" t="s">
         <v>231</v>
       </c>
-      <c r="B9" s="33">
+      <c r="B9" s="32">
         <f>B5*B6*B8</f>
         <v>10131.80576923077</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="D9" s="5" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A10" s="6" t="s">
+    <row r="10" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="5" t="s">
         <v>233</v>
       </c>
-      <c r="B10" s="35">
+      <c r="B10" s="33">
         <f>B5*12</f>
         <v>9480</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A12" s="7" t="s">
+    <row r="11" spans="1:8" ht="14.5" x14ac:dyDescent="0.35"/>
+    <row r="12" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="11" t="s">
         <v>234</v>
       </c>
-      <c r="B12" s="10"/>
-      <c r="C12" s="10"/>
-      <c r="D12" s="10"/>
-      <c r="E12" s="10"/>
-      <c r="F12" s="10"/>
-      <c r="G12" s="10"/>
-      <c r="H12" s="10"/>
-    </row>
-    <row r="13" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A13" s="6" t="s">
+      <c r="B12" s="2"/>
+      <c r="C12" s="2"/>
+      <c r="D12" s="2"/>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
+      <c r="G12" s="2"/>
+      <c r="H12" s="2"/>
+    </row>
+    <row r="13" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="5" t="s">
         <v>235</v>
       </c>
-      <c r="B13" s="23">
+      <c r="B13" s="25">
         <v>500000</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="D13" s="5" t="s">
         <v>236</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A14" s="6" t="s">
+    <row r="14" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="5" t="s">
         <v>237</v>
       </c>
-      <c r="B14" s="14">
+      <c r="B14" s="13">
         <v>250</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="C14" s="5" t="s">
         <v>238</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A15" s="6" t="s">
+    <row r="15" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="5" t="s">
         <v>239</v>
       </c>
-      <c r="B15" s="17">
+      <c r="B15" s="15">
         <f>IF(B10=0,0,B13/B10)</f>
         <v>52.742616033755276</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A16" s="12" t="s">
+    <row r="16" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="6" t="s">
         <v>240</v>
       </c>
-      <c r="B16" s="36">
+      <c r="B16" s="34">
         <f>IF(B14=0,0,B15/B14)</f>
         <v>0.2109704641350211</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C16" s="5" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A17" s="6" t="s">
+    <row r="17" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="5" t="s">
         <v>242</v>
       </c>
       <c r="B17" s="8" t="str">
@@ -7638,60 +7613,61 @@
         <v>KHẢ THI về mặt số học</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A19" s="7" t="s">
+    <row r="18" spans="1:8" ht="14.5" x14ac:dyDescent="0.35"/>
+    <row r="19" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="11" t="s">
         <v>243</v>
       </c>
-      <c r="B19" s="10"/>
-      <c r="C19" s="10"/>
-      <c r="D19" s="10"/>
-      <c r="E19" s="10"/>
-      <c r="F19" s="10"/>
-      <c r="G19" s="10"/>
-      <c r="H19" s="10"/>
-    </row>
-    <row r="20" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A20" s="6" t="s">
+      <c r="B19" s="2"/>
+      <c r="C19" s="2"/>
+      <c r="D19" s="2"/>
+      <c r="E19" s="2"/>
+      <c r="F19" s="2"/>
+      <c r="G19" s="2"/>
+      <c r="H19" s="2"/>
+    </row>
+    <row r="20" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="5" t="s">
         <v>244</v>
       </c>
-      <c r="B20" s="23">
+      <c r="B20" s="25">
         <v>8000</v>
       </c>
-      <c r="D20" s="3" t="s">
+      <c r="D20" s="5" t="s">
         <v>245</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="6" t="s">
+      <c r="A21" s="5" t="s">
         <v>246</v>
       </c>
-      <c r="B21" s="15">
+      <c r="B21" s="14">
         <v>0.25</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="6" t="s">
+      <c r="A22" s="5" t="s">
         <v>247</v>
       </c>
-      <c r="B22" s="35">
+      <c r="B22" s="33">
         <f>IF(B21=0,0,B20/B21)</f>
         <v>32000</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="12" t="s">
+      <c r="A23" s="6" t="s">
         <v>248</v>
       </c>
-      <c r="B23" s="37">
+      <c r="B23" s="35">
         <f>IF(B9=0,0,B22/B9)</f>
         <v>3.1583708500591907</v>
       </c>
-      <c r="D23" s="3" t="s">
+      <c r="D23" s="5" t="s">
         <v>249</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="6" t="s">
+      <c r="A24" s="5" t="s">
         <v>167</v>
       </c>
       <c r="B24" s="8" t="str">
@@ -7701,200 +7677,200 @@
     </row>
     <row r="25" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="26" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="7" t="s">
+      <c r="A26" s="11" t="s">
         <v>250</v>
       </c>
-      <c r="B26" s="10"/>
-      <c r="C26" s="10"/>
-      <c r="D26" s="10"/>
-      <c r="E26" s="10"/>
-      <c r="F26" s="10"/>
-      <c r="G26" s="10"/>
-      <c r="H26" s="10"/>
+      <c r="B26" s="2"/>
+      <c r="C26" s="2"/>
+      <c r="D26" s="2"/>
+      <c r="E26" s="2"/>
+      <c r="F26" s="2"/>
+      <c r="G26" s="2"/>
+      <c r="H26" s="2"/>
     </row>
     <row r="27" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="25" t="s">
+      <c r="A27" s="28" t="s">
         <v>251</v>
       </c>
-      <c r="B27" s="25" t="s">
+      <c r="B27" s="28" t="s">
         <v>252</v>
       </c>
-      <c r="C27" s="25" t="s">
+      <c r="C27" s="28" t="s">
         <v>253</v>
       </c>
-      <c r="D27" s="25" t="s">
+      <c r="D27" s="28" t="s">
         <v>254</v>
       </c>
     </row>
     <row r="28" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="6" t="s">
+      <c r="A28" s="5" t="s">
         <v>255</v>
       </c>
-      <c r="B28" s="13">
+      <c r="B28" s="12">
         <v>2</v>
       </c>
-      <c r="C28" s="13">
+      <c r="C28" s="12">
         <v>2</v>
       </c>
-      <c r="D28" s="13">
+      <c r="D28" s="12">
         <v>5</v>
       </c>
     </row>
     <row r="29" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="6" t="s">
+      <c r="A29" s="5" t="s">
         <v>256</v>
       </c>
-      <c r="B29" s="13">
+      <c r="B29" s="12">
         <v>2</v>
       </c>
-      <c r="C29" s="13">
+      <c r="C29" s="12">
         <v>4</v>
       </c>
-      <c r="D29" s="13">
+      <c r="D29" s="12">
         <v>5</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="6" t="s">
+      <c r="A30" s="5" t="s">
         <v>257</v>
       </c>
-      <c r="B30" s="13">
+      <c r="B30" s="12">
         <v>3</v>
       </c>
-      <c r="C30" s="13">
+      <c r="C30" s="12">
         <v>2</v>
       </c>
-      <c r="D30" s="13">
+      <c r="D30" s="12">
         <v>4</v>
       </c>
     </row>
     <row r="31" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="6" t="s">
+      <c r="A31" s="5" t="s">
         <v>258</v>
       </c>
-      <c r="B31" s="13">
+      <c r="B31" s="12">
         <v>3</v>
       </c>
-      <c r="C31" s="13">
+      <c r="C31" s="12">
         <v>2</v>
       </c>
-      <c r="D31" s="13">
+      <c r="D31" s="12">
         <v>5</v>
       </c>
     </row>
     <row r="32" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="6" t="s">
+      <c r="A32" s="5" t="s">
         <v>259</v>
       </c>
-      <c r="B32" s="13">
+      <c r="B32" s="12">
         <v>3</v>
       </c>
-      <c r="C32" s="13">
+      <c r="C32" s="12">
         <v>4</v>
       </c>
-      <c r="D32" s="13">
+      <c r="D32" s="12">
         <v>5</v>
       </c>
     </row>
     <row r="33" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A33" s="6" t="s">
+      <c r="A33" s="5" t="s">
         <v>260</v>
       </c>
-      <c r="B33" s="13">
+      <c r="B33" s="12">
         <v>3</v>
       </c>
-      <c r="C33" s="13">
+      <c r="C33" s="12">
         <v>3</v>
       </c>
-      <c r="D33" s="13">
+      <c r="D33" s="12">
         <v>5</v>
       </c>
     </row>
     <row r="34" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="12" t="s">
+      <c r="A34" s="6" t="s">
         <v>261</v>
       </c>
-      <c r="B34" s="24">
+      <c r="B34" s="31">
         <f>SUM(B28:B33)</f>
         <v>16</v>
       </c>
-      <c r="C34" s="24">
+      <c r="C34" s="31">
         <f>SUM(C28:C33)</f>
         <v>17</v>
       </c>
-      <c r="D34" s="24">
+      <c r="D34" s="31">
         <f>SUM(D28:D33)</f>
         <v>29</v>
       </c>
     </row>
     <row r="35" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="12" t="s">
+      <c r="A35" s="6" t="s">
         <v>262</v>
       </c>
-      <c r="B35" s="24" t="str">
+      <c r="B35" s="31" t="str">
         <f>IF(AND(B34&gt;=C34,B34&gt;=D34),"PLG",IF(C34&gt;=D34,"Sales-Led","Partner-Led"))</f>
         <v>Partner-Led</v>
       </c>
     </row>
     <row r="36" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="37" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="7" t="s">
+      <c r="A37" s="11" t="s">
         <v>263</v>
       </c>
-      <c r="B37" s="10"/>
-      <c r="C37" s="10"/>
-      <c r="D37" s="10"/>
-      <c r="E37" s="10"/>
-      <c r="F37" s="10"/>
-      <c r="G37" s="10"/>
-      <c r="H37" s="10"/>
+      <c r="B37" s="2"/>
+      <c r="C37" s="2"/>
+      <c r="D37" s="2"/>
+      <c r="E37" s="2"/>
+      <c r="F37" s="2"/>
+      <c r="G37" s="2"/>
+      <c r="H37" s="2"/>
     </row>
     <row r="38" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="6" t="s">
+      <c r="A38" s="5" t="s">
         <v>264</v>
       </c>
-      <c r="B38" s="5" t="s">
+      <c r="B38" s="7" t="s">
         <v>254</v>
       </c>
-      <c r="D38" s="3" t="s">
+      <c r="D38" s="5" t="s">
         <v>265</v>
       </c>
     </row>
     <row r="39" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="6" t="s">
+      <c r="A39" s="5" t="s">
         <v>266</v>
       </c>
-      <c r="B39" s="5" t="s">
+      <c r="B39" s="7" t="s">
         <v>267</v>
       </c>
-      <c r="D39" s="3" t="s">
+      <c r="D39" s="5" t="s">
         <v>268</v>
       </c>
     </row>
     <row r="40" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A40" s="6" t="s">
+      <c r="A40" s="5" t="s">
         <v>269</v>
       </c>
-      <c r="B40" s="5" t="s">
+      <c r="B40" s="7" t="s">
         <v>270</v>
       </c>
     </row>
     <row r="41" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A41" s="6" t="s">
+      <c r="A41" s="5" t="s">
         <v>271</v>
       </c>
-      <c r="B41" s="5" t="s">
+      <c r="B41" s="7" t="s">
         <v>272</v>
       </c>
     </row>
     <row r="42" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A42" s="6" t="s">
+      <c r="A42" s="5" t="s">
         <v>273</v>
       </c>
-      <c r="B42" s="5" t="s">
+      <c r="B42" s="7" t="s">
         <v>274</v>
       </c>
-      <c r="D42" s="3" t="s">
+      <c r="D42" s="5" t="s">
         <v>275</v>
       </c>
     </row>
@@ -8878,312 +8854,315 @@
     <col min="9" max="26" width="8.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="4" t="s">
         <v>276</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-    </row>
-    <row r="2" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A2" s="3" t="s">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+    </row>
+    <row r="2" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="5" t="s">
         <v>277</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A4" s="7" t="s">
+    <row r="3" spans="1:8" ht="14.5" x14ac:dyDescent="0.35"/>
+    <row r="4" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="11" t="s">
         <v>278</v>
       </c>
-      <c r="B4" s="10"/>
-      <c r="C4" s="10"/>
-      <c r="D4" s="10"/>
-      <c r="E4" s="10"/>
-      <c r="F4" s="10"/>
-      <c r="G4" s="10"/>
-      <c r="H4" s="10"/>
-    </row>
-    <row r="5" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A5" s="6" t="s">
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
+    </row>
+    <row r="5" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="5" t="s">
         <v>279</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="7" t="s">
         <v>280</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A6" s="6" t="s">
+    <row r="6" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="5" t="s">
         <v>281</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="7" t="s">
         <v>282</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A7" s="6" t="s">
+    <row r="7" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="5" t="s">
         <v>283</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="7" t="s">
         <v>284</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A8" s="6" t="s">
+    <row r="8" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="5" t="s">
         <v>285</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="7" t="s">
         <v>286</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="5" t="s">
         <v>287</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A10" s="7" t="s">
+    <row r="9" spans="1:8" ht="14.5" x14ac:dyDescent="0.35"/>
+    <row r="10" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="11" t="s">
         <v>288</v>
       </c>
-      <c r="B10" s="10"/>
-      <c r="C10" s="10"/>
-      <c r="D10" s="10"/>
-      <c r="E10" s="10"/>
-      <c r="F10" s="10"/>
-      <c r="G10" s="10"/>
-      <c r="H10" s="10"/>
-    </row>
-    <row r="11" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A11" s="25"/>
-      <c r="B11" s="25" t="s">
+      <c r="B10" s="2"/>
+      <c r="C10" s="2"/>
+      <c r="D10" s="2"/>
+      <c r="E10" s="2"/>
+      <c r="F10" s="2"/>
+      <c r="G10" s="2"/>
+      <c r="H10" s="2"/>
+    </row>
+    <row r="11" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="3"/>
+      <c r="B11" s="28" t="s">
         <v>289</v>
       </c>
-      <c r="C11" s="25" t="s">
+      <c r="C11" s="28" t="s">
         <v>290</v>
       </c>
-      <c r="D11" s="25" t="s">
+      <c r="D11" s="28" t="s">
         <v>291</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="6" t="s">
+      <c r="A12" s="5" t="s">
         <v>292</v>
       </c>
-      <c r="B12" s="39" t="s">
+      <c r="B12" s="36" t="s">
         <v>293</v>
       </c>
-      <c r="C12" s="39" t="s">
+      <c r="C12" s="36" t="s">
         <v>294</v>
       </c>
-      <c r="D12" s="39" t="s">
+      <c r="D12" s="36" t="s">
         <v>295</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="6" t="s">
+      <c r="A13" s="5" t="s">
         <v>296</v>
       </c>
-      <c r="B13" s="39" t="s">
+      <c r="B13" s="36" t="s">
         <v>297</v>
       </c>
-      <c r="C13" s="39" t="s">
+      <c r="C13" s="36" t="s">
         <v>298</v>
       </c>
-      <c r="D13" s="39" t="s">
+      <c r="D13" s="36" t="s">
         <v>299</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="6" t="s">
+      <c r="A14" s="5" t="s">
         <v>300</v>
       </c>
-      <c r="B14" s="39" t="s">
+      <c r="B14" s="36" t="s">
         <v>301</v>
       </c>
-      <c r="C14" s="39" t="s">
+      <c r="C14" s="36" t="s">
         <v>302</v>
       </c>
-      <c r="D14" s="39" t="s">
+      <c r="D14" s="36" t="s">
         <v>303</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="6" t="s">
+      <c r="A15" s="5" t="s">
         <v>304</v>
       </c>
-      <c r="B15" s="39" t="s">
+      <c r="B15" s="36" t="s">
         <v>305</v>
       </c>
-      <c r="C15" s="39" t="s">
+      <c r="C15" s="36" t="s">
         <v>306</v>
       </c>
-      <c r="D15" s="39" t="s">
+      <c r="D15" s="36" t="s">
         <v>307</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="6" t="s">
+      <c r="A16" s="5" t="s">
         <v>308</v>
       </c>
-      <c r="B16" s="39" t="s">
+      <c r="B16" s="36" t="s">
         <v>309</v>
       </c>
-      <c r="C16" s="39" t="s">
+      <c r="C16" s="36" t="s">
         <v>310</v>
       </c>
-      <c r="D16" s="39" t="s">
+      <c r="D16" s="36" t="s">
         <v>311</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="6" t="s">
+      <c r="A17" s="5" t="s">
         <v>312</v>
       </c>
-      <c r="B17" s="39" t="s">
+      <c r="B17" s="36" t="s">
         <v>313</v>
       </c>
-      <c r="C17" s="39" t="s">
+      <c r="C17" s="36" t="s">
         <v>314</v>
       </c>
-      <c r="D17" s="39" t="s">
+      <c r="D17" s="36" t="s">
         <v>315</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="6" t="s">
+      <c r="A18" s="5" t="s">
         <v>316</v>
       </c>
-      <c r="B18" s="39" t="s">
+      <c r="B18" s="36" t="s">
         <v>317</v>
       </c>
-      <c r="C18" s="39" t="s">
+      <c r="C18" s="36" t="s">
         <v>318</v>
       </c>
-      <c r="D18" s="39" t="s">
+      <c r="D18" s="36" t="s">
         <v>319</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A19" s="3" t="s">
+    <row r="19" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="5" t="s">
         <v>320</v>
       </c>
     </row>
+    <row r="20" spans="1:8" ht="14.5" x14ac:dyDescent="0.35"/>
     <row r="21" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="7" t="s">
+      <c r="A21" s="11" t="s">
         <v>321</v>
       </c>
-      <c r="B21" s="10"/>
-      <c r="C21" s="10"/>
-      <c r="D21" s="10"/>
-      <c r="E21" s="10"/>
-      <c r="F21" s="10"/>
-      <c r="G21" s="10"/>
-      <c r="H21" s="10"/>
+      <c r="B21" s="2"/>
+      <c r="C21" s="2"/>
+      <c r="D21" s="2"/>
+      <c r="E21" s="2"/>
+      <c r="F21" s="2"/>
+      <c r="G21" s="2"/>
+      <c r="H21" s="2"/>
     </row>
     <row r="22" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="25" t="s">
+      <c r="A22" s="28" t="s">
         <v>322</v>
       </c>
-      <c r="B22" s="25" t="s">
+      <c r="B22" s="28" t="s">
         <v>323</v>
       </c>
-      <c r="C22" s="25" t="s">
+      <c r="C22" s="28" t="s">
         <v>324</v>
       </c>
-      <c r="D22" s="25" t="s">
+      <c r="D22" s="28" t="s">
         <v>325</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="6" t="s">
+      <c r="A23" s="5" t="s">
         <v>326</v>
       </c>
-      <c r="B23" s="39" t="s">
+      <c r="B23" s="36" t="s">
         <v>270</v>
       </c>
-      <c r="C23" s="39" t="s">
+      <c r="C23" s="36" t="s">
         <v>327</v>
       </c>
-      <c r="D23" s="39" t="s">
+      <c r="D23" s="36" t="s">
         <v>328</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="6" t="s">
+      <c r="A24" s="5" t="s">
         <v>329</v>
       </c>
-      <c r="B24" s="39" t="s">
+      <c r="B24" s="36" t="s">
         <v>270</v>
       </c>
-      <c r="C24" s="39" t="s">
+      <c r="C24" s="36" t="s">
         <v>330</v>
       </c>
-      <c r="D24" s="39" t="s">
+      <c r="D24" s="36" t="s">
         <v>331</v>
       </c>
     </row>
     <row r="25" spans="1:8" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="6" t="s">
+      <c r="A25" s="5" t="s">
         <v>332</v>
       </c>
-      <c r="B25" s="39" t="s">
+      <c r="B25" s="36" t="s">
         <v>333</v>
       </c>
-      <c r="C25" s="39" t="s">
+      <c r="C25" s="36" t="s">
         <v>334</v>
       </c>
-      <c r="D25" s="39" t="s">
+      <c r="D25" s="36" t="s">
         <v>335</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="3" t="s">
+      <c r="A26" s="5" t="s">
         <v>336</v>
       </c>
     </row>
     <row r="27" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="28" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="7" t="s">
+      <c r="A28" s="11" t="s">
         <v>337</v>
       </c>
-      <c r="B28" s="10"/>
-      <c r="C28" s="10"/>
-      <c r="D28" s="10"/>
-      <c r="E28" s="10"/>
-      <c r="F28" s="10"/>
-      <c r="G28" s="10"/>
-      <c r="H28" s="10"/>
+      <c r="B28" s="2"/>
+      <c r="C28" s="2"/>
+      <c r="D28" s="2"/>
+      <c r="E28" s="2"/>
+      <c r="F28" s="2"/>
+      <c r="G28" s="2"/>
+      <c r="H28" s="2"/>
     </row>
     <row r="29" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="6" t="s">
+      <c r="A29" s="5" t="s">
         <v>338</v>
       </c>
-      <c r="B29" s="5" t="s">
+      <c r="B29" s="7" t="s">
         <v>339</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="6" t="s">
+      <c r="A30" s="5" t="s">
         <v>340</v>
       </c>
-      <c r="B30" s="5" t="s">
+      <c r="B30" s="7" t="s">
         <v>339</v>
       </c>
     </row>
     <row r="31" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="6" t="s">
+      <c r="A31" s="5" t="s">
         <v>341</v>
       </c>
-      <c r="B31" s="5" t="s">
+      <c r="B31" s="7" t="s">
         <v>339</v>
       </c>
     </row>
     <row r="32" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="6" t="s">
+      <c r="A32" s="5" t="s">
         <v>342</v>
       </c>
-      <c r="B32" s="5">
+      <c r="B32" s="7">
         <v>0</v>
       </c>
     </row>
@@ -10175,666 +10154,667 @@
     <col min="9" max="26" width="8.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="4" t="s">
         <v>343</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-    </row>
-    <row r="2" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A2" s="3" t="s">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+    </row>
+    <row r="2" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="5" t="s">
         <v>344</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="6" t="s">
+    <row r="3" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="5" t="s">
         <v>345</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="7" t="s">
         <v>346</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="5" t="s">
         <v>347</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A5" s="40" t="s">
+    <row r="4" spans="1:8" ht="14.5" x14ac:dyDescent="0.35"/>
+    <row r="5" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="37" t="s">
         <v>348</v>
       </c>
-      <c r="B5" s="40" t="s">
+      <c r="B5" s="37" t="s">
         <v>349</v>
       </c>
-      <c r="C5" s="40" t="s">
+      <c r="C5" s="37" t="s">
         <v>350</v>
       </c>
-      <c r="D5" s="40" t="s">
+      <c r="D5" s="37" t="s">
         <v>351</v>
       </c>
-      <c r="E5" s="40" t="s">
+      <c r="E5" s="37" t="s">
         <v>352</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A6" s="41" t="s">
+    <row r="6" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="38" t="s">
         <v>124</v>
       </c>
-      <c r="B6" s="41" t="s">
+      <c r="B6" s="38" t="s">
         <v>353</v>
       </c>
-      <c r="C6" s="41" t="s">
+      <c r="C6" s="38" t="s">
         <v>354</v>
       </c>
-      <c r="D6" s="41" t="s">
+      <c r="D6" s="38" t="s">
         <v>355</v>
       </c>
-      <c r="E6" s="42" t="s">
+      <c r="E6" s="39" t="s">
         <v>356</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A7" s="41" t="s">
+    <row r="7" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="38" t="s">
         <v>124</v>
       </c>
-      <c r="B7" s="41" t="s">
+      <c r="B7" s="38" t="s">
         <v>357</v>
       </c>
-      <c r="C7" s="41" t="s">
+      <c r="C7" s="38" t="s">
         <v>358</v>
       </c>
-      <c r="D7" s="41" t="s">
+      <c r="D7" s="38" t="s">
         <v>355</v>
       </c>
-      <c r="E7" s="42" t="s">
+      <c r="E7" s="39" t="s">
         <v>356</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A8" s="41" t="s">
+    <row r="8" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="38" t="s">
         <v>124</v>
       </c>
-      <c r="B8" s="41" t="s">
+      <c r="B8" s="38" t="s">
         <v>359</v>
       </c>
-      <c r="C8" s="41" t="s">
+      <c r="C8" s="38" t="s">
         <v>360</v>
       </c>
-      <c r="D8" s="41" t="s">
+      <c r="D8" s="38" t="s">
         <v>355</v>
       </c>
-      <c r="E8" s="42" t="s">
+      <c r="E8" s="39" t="s">
         <v>356</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A9" s="41" t="s">
+    <row r="9" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="38" t="s">
         <v>124</v>
       </c>
-      <c r="B9" s="41" t="s">
+      <c r="B9" s="38" t="s">
         <v>361</v>
       </c>
-      <c r="C9" s="41" t="s">
+      <c r="C9" s="38" t="s">
         <v>362</v>
       </c>
-      <c r="D9" s="41" t="s">
+      <c r="D9" s="38" t="s">
         <v>363</v>
       </c>
-      <c r="E9" s="42" t="s">
+      <c r="E9" s="39" t="s">
         <v>356</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="24" x14ac:dyDescent="0.35">
-      <c r="A10" s="41" t="s">
+    <row r="10" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="38" t="s">
         <v>124</v>
       </c>
-      <c r="B10" s="41" t="s">
+      <c r="B10" s="38" t="s">
         <v>364</v>
       </c>
-      <c r="C10" s="41" t="s">
+      <c r="C10" s="38" t="s">
         <v>365</v>
       </c>
-      <c r="D10" s="41" t="s">
+      <c r="D10" s="38" t="s">
         <v>355</v>
       </c>
-      <c r="E10" s="42" t="s">
+      <c r="E10" s="39" t="s">
         <v>366</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A11" s="41" t="s">
+    <row r="11" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="38" t="s">
         <v>124</v>
       </c>
-      <c r="B11" s="41" t="s">
+      <c r="B11" s="38" t="s">
         <v>367</v>
       </c>
-      <c r="C11" s="41" t="s">
+      <c r="C11" s="38" t="s">
         <v>368</v>
       </c>
-      <c r="D11" s="41" t="s">
+      <c r="D11" s="38" t="s">
         <v>355</v>
       </c>
-      <c r="E11" s="42" t="s">
+      <c r="E11" s="39" t="s">
         <v>369</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A12" s="41" t="s">
+    <row r="12" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="38" t="s">
         <v>124</v>
       </c>
-      <c r="B12" s="41" t="s">
+      <c r="B12" s="38" t="s">
         <v>370</v>
       </c>
-      <c r="C12" s="41" t="s">
+      <c r="C12" s="38" t="s">
         <v>371</v>
       </c>
-      <c r="D12" s="41" t="s">
+      <c r="D12" s="38" t="s">
         <v>363</v>
       </c>
-      <c r="E12" s="42" t="s">
+      <c r="E12" s="39" t="s">
         <v>369</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A13" s="41" t="s">
+    <row r="13" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="38" t="s">
         <v>124</v>
       </c>
-      <c r="B13" s="41" t="s">
+      <c r="B13" s="38" t="s">
         <v>372</v>
       </c>
-      <c r="C13" s="41" t="s">
+      <c r="C13" s="38" t="s">
         <v>373</v>
       </c>
-      <c r="D13" s="41" t="s">
+      <c r="D13" s="38" t="s">
         <v>355</v>
       </c>
-      <c r="E13" s="42" t="s">
+      <c r="E13" s="39" t="s">
         <v>374</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="24" x14ac:dyDescent="0.35">
-      <c r="A14" s="41" t="s">
+    <row r="14" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="38" t="s">
         <v>124</v>
       </c>
-      <c r="B14" s="41" t="s">
+      <c r="B14" s="38" t="s">
         <v>375</v>
       </c>
-      <c r="C14" s="41" t="s">
+      <c r="C14" s="38" t="s">
         <v>376</v>
       </c>
-      <c r="D14" s="41" t="s">
+      <c r="D14" s="38" t="s">
         <v>355</v>
       </c>
-      <c r="E14" s="42" t="s">
+      <c r="E14" s="39" t="s">
         <v>377</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A15" s="41" t="s">
+    <row r="15" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="38" t="s">
         <v>378</v>
       </c>
-      <c r="B15" s="41" t="s">
+      <c r="B15" s="38" t="s">
         <v>379</v>
       </c>
-      <c r="C15" s="41" t="s">
+      <c r="C15" s="38" t="s">
         <v>380</v>
       </c>
-      <c r="D15" s="41" t="s">
+      <c r="D15" s="38" t="s">
         <v>381</v>
       </c>
-      <c r="E15" s="42" t="s">
+      <c r="E15" s="39" t="s">
         <v>382</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A16" s="41" t="s">
+    <row r="16" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="38" t="s">
         <v>378</v>
       </c>
-      <c r="B16" s="41" t="s">
+      <c r="B16" s="38" t="s">
         <v>383</v>
       </c>
-      <c r="C16" s="41" t="s">
+      <c r="C16" s="38" t="s">
         <v>384</v>
       </c>
-      <c r="D16" s="41" t="s">
+      <c r="D16" s="38" t="s">
         <v>381</v>
       </c>
-      <c r="E16" s="42" t="s">
+      <c r="E16" s="39" t="s">
         <v>385</v>
       </c>
     </row>
-    <row r="17" spans="1:5" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A17" s="41" t="s">
+    <row r="17" spans="1:5" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="38" t="s">
         <v>378</v>
       </c>
-      <c r="B17" s="41" t="s">
+      <c r="B17" s="38" t="s">
         <v>386</v>
       </c>
-      <c r="C17" s="41" t="s">
+      <c r="C17" s="38" t="s">
         <v>387</v>
       </c>
-      <c r="D17" s="41" t="s">
+      <c r="D17" s="38" t="s">
         <v>381</v>
       </c>
-      <c r="E17" s="42" t="s">
+      <c r="E17" s="39" t="s">
         <v>388</v>
       </c>
     </row>
-    <row r="18" spans="1:5" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A18" s="41" t="s">
+    <row r="18" spans="1:5" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="38" t="s">
         <v>378</v>
       </c>
-      <c r="B18" s="41" t="s">
+      <c r="B18" s="38" t="s">
         <v>389</v>
       </c>
-      <c r="C18" s="41" t="s">
+      <c r="C18" s="38" t="s">
         <v>390</v>
       </c>
-      <c r="D18" s="41" t="s">
+      <c r="D18" s="38" t="s">
         <v>381</v>
       </c>
-      <c r="E18" s="42" t="s">
+      <c r="E18" s="39" t="s">
         <v>369</v>
       </c>
     </row>
-    <row r="19" spans="1:5" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A19" s="41" t="s">
+    <row r="19" spans="1:5" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="38" t="s">
         <v>391</v>
       </c>
-      <c r="B19" s="41" t="s">
+      <c r="B19" s="38" t="s">
         <v>392</v>
       </c>
-      <c r="C19" s="41" t="s">
+      <c r="C19" s="38" t="s">
         <v>393</v>
       </c>
-      <c r="D19" s="41" t="s">
+      <c r="D19" s="38" t="s">
         <v>394</v>
       </c>
-      <c r="E19" s="42" t="s">
+      <c r="E19" s="39" t="s">
         <v>395</v>
       </c>
     </row>
-    <row r="20" spans="1:5" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A20" s="41" t="s">
+    <row r="20" spans="1:5" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="38" t="s">
         <v>391</v>
       </c>
-      <c r="B20" s="41" t="s">
+      <c r="B20" s="38" t="s">
         <v>396</v>
       </c>
-      <c r="C20" s="41" t="s">
+      <c r="C20" s="38" t="s">
         <v>397</v>
       </c>
-      <c r="D20" s="41" t="s">
+      <c r="D20" s="38" t="s">
         <v>394</v>
       </c>
-      <c r="E20" s="42" t="s">
+      <c r="E20" s="39" t="s">
         <v>369</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="41" t="s">
+      <c r="A21" s="38" t="s">
         <v>391</v>
       </c>
-      <c r="B21" s="41" t="s">
+      <c r="B21" s="38" t="s">
         <v>398</v>
       </c>
-      <c r="C21" s="41" t="s">
+      <c r="C21" s="38" t="s">
         <v>399</v>
       </c>
-      <c r="D21" s="41" t="s">
+      <c r="D21" s="38" t="s">
         <v>394</v>
       </c>
-      <c r="E21" s="42" t="s">
+      <c r="E21" s="39" t="s">
         <v>400</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="41" t="s">
+      <c r="A22" s="38" t="s">
         <v>391</v>
       </c>
-      <c r="B22" s="41" t="s">
+      <c r="B22" s="38" t="s">
         <v>401</v>
       </c>
-      <c r="C22" s="41" t="s">
+      <c r="C22" s="38" t="s">
         <v>402</v>
       </c>
-      <c r="D22" s="41" t="s">
+      <c r="D22" s="38" t="s">
         <v>394</v>
       </c>
-      <c r="E22" s="42" t="s">
+      <c r="E22" s="39" t="s">
         <v>400</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="41" t="s">
+      <c r="A23" s="38" t="s">
         <v>403</v>
       </c>
-      <c r="B23" s="41" t="s">
+      <c r="B23" s="38" t="s">
         <v>404</v>
       </c>
-      <c r="C23" s="41" t="s">
+      <c r="C23" s="38" t="s">
         <v>405</v>
       </c>
-      <c r="D23" s="41" t="s">
+      <c r="D23" s="38" t="s">
         <v>406</v>
       </c>
-      <c r="E23" s="42" t="s">
+      <c r="E23" s="39" t="s">
         <v>407</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="41" t="s">
+      <c r="A24" s="38" t="s">
         <v>408</v>
       </c>
-      <c r="B24" s="41" t="s">
+      <c r="B24" s="38" t="s">
         <v>409</v>
       </c>
-      <c r="C24" s="41" t="s">
+      <c r="C24" s="38" t="s">
         <v>410</v>
       </c>
-      <c r="D24" s="41" t="s">
+      <c r="D24" s="38" t="s">
         <v>411</v>
       </c>
-      <c r="E24" s="42" t="s">
+      <c r="E24" s="39" t="s">
         <v>412</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="41" t="s">
+      <c r="A25" s="38" t="s">
         <v>408</v>
       </c>
-      <c r="B25" s="41" t="s">
+      <c r="B25" s="38" t="s">
         <v>413</v>
       </c>
-      <c r="C25" s="41" t="s">
+      <c r="C25" s="38" t="s">
         <v>414</v>
       </c>
-      <c r="D25" s="41" t="s">
+      <c r="D25" s="38" t="s">
         <v>411</v>
       </c>
-      <c r="E25" s="42" t="s">
+      <c r="E25" s="39" t="s">
         <v>415</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="41" t="s">
+      <c r="A26" s="38" t="s">
         <v>408</v>
       </c>
-      <c r="B26" s="41" t="s">
+      <c r="B26" s="38" t="s">
         <v>416</v>
       </c>
-      <c r="C26" s="41" t="s">
+      <c r="C26" s="38" t="s">
         <v>417</v>
       </c>
-      <c r="D26" s="41" t="s">
+      <c r="D26" s="38" t="s">
         <v>363</v>
       </c>
-      <c r="E26" s="42" t="s">
+      <c r="E26" s="39" t="s">
         <v>418</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="41" t="s">
+      <c r="A27" s="38" t="s">
         <v>419</v>
       </c>
-      <c r="B27" s="41" t="s">
+      <c r="B27" s="38" t="s">
         <v>420</v>
       </c>
-      <c r="C27" s="41" t="s">
+      <c r="C27" s="38" t="s">
         <v>421</v>
       </c>
-      <c r="D27" s="41" t="s">
+      <c r="D27" s="38" t="s">
         <v>422</v>
       </c>
-      <c r="E27" s="42" t="s">
+      <c r="E27" s="39" t="s">
         <v>423</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="41" t="s">
+      <c r="A28" s="38" t="s">
         <v>419</v>
       </c>
-      <c r="B28" s="41" t="s">
+      <c r="B28" s="38" t="s">
         <v>424</v>
       </c>
-      <c r="C28" s="41" t="s">
+      <c r="C28" s="38" t="s">
         <v>425</v>
       </c>
-      <c r="D28" s="41" t="s">
+      <c r="D28" s="38" t="s">
         <v>422</v>
       </c>
-      <c r="E28" s="42" t="s">
+      <c r="E28" s="39" t="s">
         <v>423</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="41" t="s">
+      <c r="A29" s="38" t="s">
         <v>419</v>
       </c>
-      <c r="B29" s="41" t="s">
+      <c r="B29" s="38" t="s">
         <v>426</v>
       </c>
-      <c r="C29" s="41" t="s">
+      <c r="C29" s="38" t="s">
         <v>427</v>
       </c>
-      <c r="D29" s="41" t="s">
+      <c r="D29" s="38" t="s">
         <v>428</v>
       </c>
-      <c r="E29" s="42" t="s">
+      <c r="E29" s="39" t="s">
         <v>429</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="41" t="s">
+      <c r="A30" s="38" t="s">
         <v>419</v>
       </c>
-      <c r="B30" s="41" t="s">
+      <c r="B30" s="38" t="s">
         <v>430</v>
       </c>
-      <c r="C30" s="41" t="s">
+      <c r="C30" s="38" t="s">
         <v>431</v>
       </c>
-      <c r="D30" s="41" t="s">
+      <c r="D30" s="38" t="s">
         <v>432</v>
       </c>
-      <c r="E30" s="42" t="s">
+      <c r="E30" s="39" t="s">
         <v>433</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="41" t="s">
+      <c r="A31" s="38" t="s">
         <v>419</v>
       </c>
-      <c r="B31" s="41" t="s">
+      <c r="B31" s="38" t="s">
         <v>434</v>
       </c>
-      <c r="C31" s="41" t="s">
+      <c r="C31" s="38" t="s">
         <v>435</v>
       </c>
-      <c r="D31" s="41" t="s">
+      <c r="D31" s="38" t="s">
         <v>436</v>
       </c>
-      <c r="E31" s="42" t="s">
+      <c r="E31" s="39" t="s">
         <v>433</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="41" t="s">
+      <c r="A32" s="38" t="s">
         <v>419</v>
       </c>
-      <c r="B32" s="41" t="s">
+      <c r="B32" s="38" t="s">
         <v>437</v>
       </c>
-      <c r="C32" s="41" t="s">
+      <c r="C32" s="38" t="s">
         <v>438</v>
       </c>
-      <c r="D32" s="41" t="s">
+      <c r="D32" s="38" t="s">
         <v>432</v>
       </c>
-      <c r="E32" s="42" t="s">
+      <c r="E32" s="39" t="s">
         <v>439</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A33" s="41" t="s">
+      <c r="A33" s="38" t="s">
         <v>419</v>
       </c>
-      <c r="B33" s="41" t="s">
+      <c r="B33" s="38" t="s">
         <v>440</v>
       </c>
-      <c r="C33" s="41" t="s">
+      <c r="C33" s="38" t="s">
         <v>441</v>
       </c>
-      <c r="D33" s="41" t="s">
+      <c r="D33" s="38" t="s">
         <v>442</v>
       </c>
-      <c r="E33" s="42" t="s">
+      <c r="E33" s="39" t="s">
         <v>439</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="41" t="s">
+      <c r="A34" s="38" t="s">
         <v>419</v>
       </c>
-      <c r="B34" s="41" t="s">
+      <c r="B34" s="38" t="s">
         <v>443</v>
       </c>
-      <c r="C34" s="41" t="s">
+      <c r="C34" s="38" t="s">
         <v>444</v>
       </c>
-      <c r="D34" s="41" t="s">
+      <c r="D34" s="38" t="s">
         <v>445</v>
       </c>
-      <c r="E34" s="42" t="s">
+      <c r="E34" s="39" t="s">
         <v>446</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="41" t="s">
+      <c r="A35" s="38" t="s">
         <v>447</v>
       </c>
-      <c r="B35" s="41" t="s">
+      <c r="B35" s="38" t="s">
         <v>448</v>
       </c>
-      <c r="C35" s="41" t="s">
+      <c r="C35" s="38" t="s">
         <v>449</v>
       </c>
-      <c r="D35" s="41" t="s">
+      <c r="D35" s="38" t="s">
         <v>450</v>
       </c>
-      <c r="E35" s="42" t="s">
+      <c r="E35" s="39" t="s">
         <v>451</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="41" t="s">
+      <c r="A36" s="38" t="s">
         <v>447</v>
       </c>
-      <c r="B36" s="41" t="s">
+      <c r="B36" s="38" t="s">
         <v>452</v>
       </c>
-      <c r="C36" s="41" t="s">
+      <c r="C36" s="38" t="s">
         <v>453</v>
       </c>
-      <c r="D36" s="41" t="s">
+      <c r="D36" s="38" t="s">
         <v>450</v>
       </c>
-      <c r="E36" s="42" t="s">
+      <c r="E36" s="39" t="s">
         <v>454</v>
       </c>
     </row>
     <row r="37" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="41" t="s">
+      <c r="A37" s="38" t="s">
         <v>447</v>
       </c>
-      <c r="B37" s="41" t="s">
+      <c r="B37" s="38" t="s">
         <v>455</v>
       </c>
-      <c r="C37" s="41" t="s">
+      <c r="C37" s="38" t="s">
         <v>456</v>
       </c>
-      <c r="D37" s="41" t="s">
+      <c r="D37" s="38" t="s">
         <v>450</v>
       </c>
-      <c r="E37" s="42" t="s">
+      <c r="E37" s="39" t="s">
         <v>457</v>
       </c>
     </row>
     <row r="38" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="41" t="s">
+      <c r="A38" s="38" t="s">
         <v>447</v>
       </c>
-      <c r="B38" s="41" t="s">
+      <c r="B38" s="38" t="s">
         <v>458</v>
       </c>
-      <c r="C38" s="41" t="s">
+      <c r="C38" s="38" t="s">
         <v>459</v>
       </c>
-      <c r="D38" s="41" t="s">
+      <c r="D38" s="38" t="s">
         <v>229</v>
       </c>
-      <c r="E38" s="42" t="s">
+      <c r="E38" s="39" t="s">
         <v>454</v>
       </c>
     </row>
     <row r="39" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="41" t="s">
+      <c r="A39" s="38" t="s">
         <v>447</v>
       </c>
-      <c r="B39" s="41" t="s">
+      <c r="B39" s="38" t="s">
         <v>460</v>
       </c>
-      <c r="C39" s="41" t="s">
+      <c r="C39" s="38" t="s">
         <v>461</v>
       </c>
-      <c r="D39" s="41" t="s">
+      <c r="D39" s="38" t="s">
         <v>462</v>
       </c>
-      <c r="E39" s="42" t="s">
+      <c r="E39" s="39" t="s">
         <v>463</v>
       </c>
     </row>
     <row r="40" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A40" s="41" t="s">
+      <c r="A40" s="38" t="s">
         <v>447</v>
       </c>
-      <c r="B40" s="41" t="s">
+      <c r="B40" s="38" t="s">
         <v>464</v>
       </c>
-      <c r="C40" s="41" t="s">
+      <c r="C40" s="38" t="s">
         <v>465</v>
       </c>
-      <c r="D40" s="41" t="s">
+      <c r="D40" s="38" t="s">
         <v>466</v>
       </c>
-      <c r="E40" s="42" t="s">
+      <c r="E40" s="39" t="s">
         <v>467</v>
       </c>
     </row>
     <row r="41" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A41" s="41" t="s">
+      <c r="A41" s="38" t="s">
         <v>447</v>
       </c>
-      <c r="B41" s="41" t="s">
+      <c r="B41" s="38" t="s">
         <v>468</v>
       </c>
-      <c r="C41" s="41" t="s">
+      <c r="C41" s="38" t="s">
         <v>469</v>
       </c>
-      <c r="D41" s="41" t="s">
+      <c r="D41" s="38" t="s">
         <v>470</v>
       </c>
-      <c r="E41" s="42" t="s">
+      <c r="E41" s="39" t="s">
         <v>471</v>
       </c>
     </row>
     <row r="42" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="43" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A43" s="3" t="s">
+      <c r="A43" s="5" t="s">
         <v>472</v>
       </c>
     </row>

</xml_diff>